<commit_message>
Update Task 2, 4
</commit_message>
<xml_diff>
--- a/Task_02/DucNVFX14814_OPPM_Plan.xlsx
+++ b/Task_02/DucNVFX14814_OPPM_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Funix\4. CC4\5. LAB301x\LAB301x_01\Task_02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5381615F-8EBD-48A3-A749-3D7D616F15B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670AA11E-5886-49BA-865E-DB3C35401B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Start" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Start!$B$2:$W$56</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Start!$B$2:$U$51</definedName>
   </definedNames>
   <calcPr calcId="152511" iterate="1" iterateCount="10000" iterateDelta="1.0000000000000001E-5"/>
   <extLst>
@@ -33,7 +33,7 @@
     <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="J59" authorId="0" shapeId="0" xr:uid="{F90B73BB-1F15-CD43-AECB-A57B7C17353B}">
+    <comment ref="J54" authorId="0" shapeId="0" xr:uid="{F90B73BB-1F15-CD43-AECB-A57B7C17353B}">
       <text>
         <r>
           <rPr>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="66">
   <si>
     <t>Sub-Objectives</t>
   </si>
@@ -128,36 +128,6 @@
   </si>
   <si>
     <t>Dev 4</t>
-  </si>
-  <si>
-    <t>Day 1</t>
-  </si>
-  <si>
-    <t>Day 2</t>
-  </si>
-  <si>
-    <t>Day 3</t>
-  </si>
-  <si>
-    <t>Day 4</t>
-  </si>
-  <si>
-    <t>Day 5</t>
-  </si>
-  <si>
-    <t>Day 6</t>
-  </si>
-  <si>
-    <t>Day 7</t>
-  </si>
-  <si>
-    <t>Day 8</t>
-  </si>
-  <si>
-    <t>Day 9</t>
-  </si>
-  <si>
-    <t>Day 10</t>
   </si>
   <si>
     <t>Primary Owner</t>
@@ -203,21 +173,9 @@
     <t>Task1c: Đặc tả Use case &amp; danh sách màn hình, hoàn thiện SRS (2 ngày)</t>
   </si>
   <si>
-    <t>Task2: Lập kế hoạch dự án OPPM_Plan (1 ngày)</t>
-  </si>
-  <si>
-    <t>Task3a: Thiết kế kiến trúc &amp; tổ chức code (2 ngày)</t>
-  </si>
-  <si>
     <t>Task4a: Thiết kế cơ sở dữ liệu - vẽ ERD (2 ngày)</t>
   </si>
   <si>
-    <t>Task4b: Nhập dữ liệu mẫu (1 ngày)</t>
-  </si>
-  <si>
-    <t>Task4c: Viết script tạo CSDL (1 ngày)</t>
-  </si>
-  <si>
     <t>Task5a: Thiết kế giao diện Đăng ký/Đăng nhập/Quản lý người dùng (2 ngày)</t>
   </si>
   <si>
@@ -269,7 +227,49 @@
     <t>Học viên không đảm bảo được thời gian làm việc -&gt; có thể làm chậm tiến độ dự án</t>
   </si>
   <si>
-    <t>Chỉ số: Tiến độ hoàn thành các Task theo đúng lịch trong OPPM_Plan.</t>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Week 7</t>
+  </si>
+  <si>
+    <t>Week 8</t>
+  </si>
+  <si>
+    <t>Lấy API dữ liệu từ trang web Xổ số Minh Ngọc, phụ thuộc vào kết quả từ trang web khác</t>
+  </si>
+  <si>
+    <t>Task4b: Viết script tạo CSDL (1 ngày)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task4c: Nhập dữ liệu mẫu (1 ngày)		</t>
+  </si>
+  <si>
+    <t>Task2: Lập kế hoạch dự án OPPM_Plan (2 ngày)</t>
+  </si>
+  <si>
+    <t>Task3: Thiết kế kiến trúc &amp; tổ chức code (2 ngày)</t>
+  </si>
+  <si>
+    <t>Chỉ số: Tiến độ hoàn thành các Task theo đúng lịch trong OPPM_Plan</t>
+  </si>
+  <si>
+    <t>Kết quả vé dò được Admin tạo thủ công và Publish hàng ngày, nên kết quả có thể chậm trễ, không cập nhật kịp thời để người dùng dò vé</t>
   </si>
 </sst>
 </file>
@@ -281,7 +281,7 @@
     <numFmt numFmtId="165" formatCode="0000"/>
     <numFmt numFmtId="166" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -395,14 +395,28 @@
       <scheme val="major"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <scheme val="major"/>
@@ -459,18 +473,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6600CC"/>
+        <fgColor rgb="FF0070C0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0070C0"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="0"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="77">
+  <borders count="83">
     <border>
       <left/>
       <right/>
@@ -831,21 +845,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="hair">
-        <color rgb="FFC0C0C0"/>
-      </left>
-      <right style="hair">
-        <color rgb="FFC0C0C0"/>
-      </right>
-      <top style="hair">
-        <color rgb="FFC0C0C0"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="FFC0C0C0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color auto="1"/>
       </left>
@@ -1025,26 +1024,6 @@
         <color indexed="22"/>
       </left>
       <right/>
-      <top/>
-      <bottom style="hair">
-        <color indexed="22"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="hair">
-        <color indexed="22"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
       <top/>
       <bottom style="hair">
         <color indexed="22"/>
@@ -1248,19 +1227,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="hair">
@@ -1448,6 +1414,142 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color indexed="22"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="22"/>
+      </left>
+      <right style="hair">
+        <color indexed="22"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="22"/>
+      </right>
+      <top style="hair">
+        <color indexed="22"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="22"/>
+      </left>
+      <right style="hair">
+        <color indexed="22"/>
+      </right>
+      <top style="hair">
+        <color indexed="22"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="22"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="22"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="22"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="22"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="22"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color indexed="22"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="22"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="22"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1462,7 +1564,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="216">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -1539,23 +1641,7 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -1574,15 +1660,15 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -1650,186 +1736,135 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="42" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="43" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="48" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="50" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -1839,45 +1874,45 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="48" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="50" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1948,7 +1983,7 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1962,47 +1997,83 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="67" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="68" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="73" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="74" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="74" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="75" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="76" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="65" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="66" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="67" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="68" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="69" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2021,26 +2092,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="66" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="73" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="74" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="75" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="76" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2116,63 +2167,95 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="65" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="17" fontId="10" fillId="0" borderId="54" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="17" fontId="10" fillId="0" borderId="51" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="17" fontId="10" fillId="0" borderId="47" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="17" fontId="10" fillId="0" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="47" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="58" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2184,36 +2267,71 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="61" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="78" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="79" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="73" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="80" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="81" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="78" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="82" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="16" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="16" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="75" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="76" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="77" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2561,20 +2679,6 @@
           <c:tx>
             <c:v>Budgeted</c:v>
           </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="tx2">
-                <a:lumMod val="20000"/>
-                <a:lumOff val="80000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln w="6350">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:spPr>
@@ -2847,13 +2951,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2901,13 +3005,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>21770</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>925285</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>642256</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2955,13 +3059,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>683079</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>1949904</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>281668</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3019,13 +3123,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>289831</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>65314</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>1583550</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3083,13 +3187,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>1265464</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>152401</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>636814</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3147,13 +3251,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>1338943</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>10888</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>908958</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>112699</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3285,13 +3389,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3339,13 +3443,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>475707</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>143692</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>947057</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>10886</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3400,13 +3504,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>21770</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>914400</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>642256</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3454,13 +3558,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>1071789</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>113392</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>1709964</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>94342</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3548,15 +3652,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>26</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>395817</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>84666</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
+      <xdr:col>26</xdr:col>
       <xdr:colOff>156634</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3611,13 +3715,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>43544</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>43543</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>620486</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3973,7 +4077,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AA64"/>
+  <dimension ref="B1:Y59"/>
   <sheetFormatPr defaultColWidth="10.1796875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
@@ -3981,28 +4085,28 @@
     <col min="6" max="6" width="21.1796875" style="1" customWidth="1"/>
     <col min="7" max="7" width="25" style="1" customWidth="1"/>
     <col min="8" max="8" width="11.36328125" style="1" customWidth="1"/>
-    <col min="9" max="18" width="5.81640625" style="1" customWidth="1"/>
-    <col min="19" max="22" width="4.81640625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="5.1796875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="1.81640625" style="1" customWidth="1"/>
-    <col min="25" max="25" width="19.26953125" style="2" customWidth="1"/>
-    <col min="26" max="26" width="9.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="16384" width="10.1796875" style="1"/>
+    <col min="9" max="16" width="5.81640625" style="1" customWidth="1"/>
+    <col min="17" max="20" width="4.81640625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="5.1796875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="1.81640625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="19.26953125" style="2" customWidth="1"/>
+    <col min="24" max="24" width="9.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="16384" width="10.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:27" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:27" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:25" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:25" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="B2" s="4"/>
       <c r="C2" s="5"/>
       <c r="D2" s="6"/>
       <c r="E2" s="7" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="8" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
@@ -4012,121 +4116,113 @@
       <c r="N2" s="10"/>
       <c r="O2" s="10"/>
       <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
       <c r="S2" s="12"/>
       <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y2" s="15"/>
-      <c r="Z2" s="16"/>
-      <c r="AA2" s="16"/>
+      <c r="U2" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="W2" s="15"/>
+      <c r="X2" s="16"/>
+      <c r="Y2" s="16"/>
     </row>
-    <row r="3" spans="2:27" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:25" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="17"/>
       <c r="D3" s="18"/>
-      <c r="E3" s="178" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="179"/>
-      <c r="G3" s="179"/>
-      <c r="H3" s="179"/>
-      <c r="I3" s="179"/>
-      <c r="J3" s="179"/>
-      <c r="K3" s="179"/>
-      <c r="L3" s="179"/>
-      <c r="M3" s="179"/>
-      <c r="N3" s="179"/>
-      <c r="O3" s="179"/>
-      <c r="P3" s="179"/>
-      <c r="Q3" s="179"/>
-      <c r="R3" s="179"/>
-      <c r="S3" s="179"/>
-      <c r="T3" s="179"/>
-      <c r="U3" s="179"/>
-      <c r="V3" s="179"/>
-      <c r="W3" s="180"/>
-      <c r="Y3" s="15"/>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="16"/>
+      <c r="E3" s="165" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="166"/>
+      <c r="G3" s="166"/>
+      <c r="H3" s="166"/>
+      <c r="I3" s="166"/>
+      <c r="J3" s="166"/>
+      <c r="K3" s="166"/>
+      <c r="L3" s="166"/>
+      <c r="M3" s="166"/>
+      <c r="N3" s="166"/>
+      <c r="O3" s="166"/>
+      <c r="P3" s="166"/>
+      <c r="Q3" s="166"/>
+      <c r="R3" s="166"/>
+      <c r="S3" s="166"/>
+      <c r="T3" s="166"/>
+      <c r="U3" s="167"/>
+      <c r="W3" s="15"/>
+      <c r="X3" s="16"/>
+      <c r="Y3" s="16"/>
     </row>
-    <row r="4" spans="2:27" s="21" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:25" s="21" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="19"/>
       <c r="C4" s="20"/>
       <c r="D4" s="20"/>
-      <c r="E4" s="181"/>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
-      <c r="H4" s="182"/>
-      <c r="I4" s="182"/>
-      <c r="J4" s="182"/>
-      <c r="K4" s="182"/>
-      <c r="L4" s="182"/>
-      <c r="M4" s="182"/>
-      <c r="N4" s="182"/>
-      <c r="O4" s="182"/>
-      <c r="P4" s="182"/>
-      <c r="Q4" s="182"/>
-      <c r="R4" s="182"/>
-      <c r="S4" s="182"/>
-      <c r="T4" s="182"/>
-      <c r="U4" s="182"/>
-      <c r="V4" s="182"/>
-      <c r="W4" s="183"/>
-      <c r="Y4" s="22"/>
-      <c r="Z4" s="23"/>
-      <c r="AA4" s="23"/>
+      <c r="E4" s="168"/>
+      <c r="F4" s="169"/>
+      <c r="G4" s="169"/>
+      <c r="H4" s="169"/>
+      <c r="I4" s="169"/>
+      <c r="J4" s="169"/>
+      <c r="K4" s="169"/>
+      <c r="L4" s="169"/>
+      <c r="M4" s="169"/>
+      <c r="N4" s="169"/>
+      <c r="O4" s="169"/>
+      <c r="P4" s="169"/>
+      <c r="Q4" s="169"/>
+      <c r="R4" s="169"/>
+      <c r="S4" s="169"/>
+      <c r="T4" s="169"/>
+      <c r="U4" s="170"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="23"/>
+      <c r="Y4" s="23"/>
     </row>
-    <row r="5" spans="2:27" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="184" t="s">
+    <row r="5" spans="2:25" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="171" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="185"/>
-      <c r="D5" s="186"/>
+      <c r="C5" s="172"/>
+      <c r="D5" s="173"/>
       <c r="E5" s="24"/>
       <c r="F5" s="25" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
-      <c r="I5" s="187" t="s">
+      <c r="I5" s="174" t="s">
         <v>2</v>
       </c>
-      <c r="J5" s="188"/>
-      <c r="K5" s="188"/>
-      <c r="L5" s="188"/>
-      <c r="M5" s="188"/>
-      <c r="N5" s="188"/>
-      <c r="O5" s="188"/>
-      <c r="P5" s="188"/>
-      <c r="Q5" s="188"/>
-      <c r="R5" s="189"/>
-      <c r="S5" s="187" t="s">
+      <c r="J5" s="175"/>
+      <c r="K5" s="175"/>
+      <c r="L5" s="175"/>
+      <c r="M5" s="175"/>
+      <c r="N5" s="175"/>
+      <c r="O5" s="175"/>
+      <c r="P5" s="175"/>
+      <c r="Q5" s="174" t="s">
         <v>3</v>
       </c>
-      <c r="T5" s="188"/>
-      <c r="U5" s="188"/>
-      <c r="V5" s="189"/>
-      <c r="W5" s="190"/>
+      <c r="R5" s="175"/>
+      <c r="S5" s="175"/>
+      <c r="T5" s="176"/>
+      <c r="U5" s="177"/>
     </row>
-    <row r="6" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B6" s="160" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="161"/>
-      <c r="D6" s="162"/>
-      <c r="E6" s="153">
+    <row r="6" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B6" s="147" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="148"/>
+      <c r="D6" s="149"/>
+      <c r="E6" s="135">
         <v>1</v>
       </c>
-      <c r="F6" s="158" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="159"/>
-      <c r="H6" s="159"/>
-      <c r="I6" s="149">
+      <c r="F6" s="145" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="146"/>
+      <c r="H6" s="146"/>
+      <c r="I6" s="132">
         <v>2</v>
       </c>
       <c r="J6" s="29"/>
@@ -4135,1650 +4231,1455 @@
       <c r="M6" s="29"/>
       <c r="N6" s="29"/>
       <c r="O6" s="29"/>
-      <c r="P6" s="29"/>
-      <c r="Q6" s="29"/>
-      <c r="R6" s="29"/>
-      <c r="S6" s="30"/>
-      <c r="T6" s="31"/>
-      <c r="U6" s="32"/>
-      <c r="V6" s="33"/>
-      <c r="W6" s="34"/>
-      <c r="Y6" s="36"/>
-      <c r="Z6" s="37"/>
-      <c r="AA6" s="37"/>
+      <c r="P6" s="203"/>
+      <c r="Q6" s="209" t="s">
+        <v>11</v>
+      </c>
+      <c r="R6" s="210"/>
+      <c r="S6" s="211"/>
+      <c r="T6" s="212"/>
+      <c r="U6" s="213"/>
+      <c r="W6" s="32"/>
+      <c r="X6" s="33"/>
+      <c r="Y6" s="33"/>
     </row>
-    <row r="7" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B7" s="163"/>
-      <c r="C7" s="164"/>
-      <c r="D7" s="165"/>
-      <c r="E7" s="154">
+    <row r="7" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="150"/>
+      <c r="C7" s="151"/>
+      <c r="D7" s="152"/>
+      <c r="E7" s="136">
         <v>2</v>
       </c>
-      <c r="F7" s="158" t="s">
+      <c r="F7" s="145" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="146"/>
+      <c r="H7" s="146"/>
+      <c r="I7" s="132">
+        <v>2</v>
+      </c>
+      <c r="J7" s="38"/>
+      <c r="K7" s="38"/>
+      <c r="L7" s="38"/>
+      <c r="M7" s="38"/>
+      <c r="N7" s="38"/>
+      <c r="O7" s="38"/>
+      <c r="P7" s="68"/>
+      <c r="Q7" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R7" s="30"/>
+      <c r="S7" s="40"/>
+      <c r="T7" s="40"/>
+      <c r="U7" s="41"/>
+      <c r="W7" s="32"/>
+      <c r="X7" s="33"/>
+      <c r="Y7" s="33"/>
+    </row>
+    <row r="8" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="150"/>
+      <c r="C8" s="151"/>
+      <c r="D8" s="152"/>
+      <c r="E8" s="136">
+        <v>3</v>
+      </c>
+      <c r="F8" s="145" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" s="146"/>
+      <c r="H8" s="146"/>
+      <c r="I8" s="133">
+        <v>1</v>
+      </c>
+      <c r="J8" s="134">
+        <v>1</v>
+      </c>
+      <c r="K8" s="47"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="47"/>
+      <c r="N8" s="47"/>
+      <c r="O8" s="47"/>
+      <c r="P8" s="50"/>
+      <c r="Q8" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R8" s="215"/>
+      <c r="S8" s="40"/>
+      <c r="T8" s="40"/>
+      <c r="U8" s="49"/>
+      <c r="W8" s="32"/>
+      <c r="X8" s="33"/>
+      <c r="Y8" s="33"/>
+    </row>
+    <row r="9" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="153"/>
+      <c r="C9" s="154"/>
+      <c r="D9" s="155"/>
+      <c r="E9" s="135">
+        <v>4</v>
+      </c>
+      <c r="F9" s="145" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" s="146"/>
+      <c r="H9" s="146"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="134">
+        <v>2</v>
+      </c>
+      <c r="K9" s="50"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="47"/>
+      <c r="O9" s="47"/>
+      <c r="P9" s="50"/>
+      <c r="Q9" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R9" s="40"/>
+      <c r="S9" s="40"/>
+      <c r="T9" s="40"/>
+      <c r="U9" s="41"/>
+      <c r="W9" s="32"/>
+      <c r="X9" s="33"/>
+      <c r="Y9" s="33"/>
+    </row>
+    <row r="10" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="156" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="157"/>
+      <c r="D10" s="158"/>
+      <c r="E10" s="135">
+        <v>5</v>
+      </c>
+      <c r="F10" s="145" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" s="146"/>
+      <c r="H10" s="146"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="134">
+        <v>2</v>
+      </c>
+      <c r="K10" s="50"/>
+      <c r="L10" s="38"/>
+      <c r="M10" s="51"/>
+      <c r="N10" s="47"/>
+      <c r="O10" s="47"/>
+      <c r="P10" s="50"/>
+      <c r="Q10" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R10" s="40"/>
+      <c r="S10" s="215"/>
+      <c r="T10" s="40"/>
+      <c r="U10" s="49"/>
+      <c r="W10" s="32"/>
+      <c r="X10" s="33"/>
+      <c r="Y10" s="33"/>
+    </row>
+    <row r="11" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B11" s="159"/>
+      <c r="C11" s="160"/>
+      <c r="D11" s="161"/>
+      <c r="E11" s="135">
+        <v>6</v>
+      </c>
+      <c r="F11" s="145" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="146"/>
+      <c r="H11" s="146"/>
+      <c r="I11" s="46"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="134">
+        <v>2</v>
+      </c>
+      <c r="L11" s="38"/>
+      <c r="M11" s="38"/>
+      <c r="N11" s="47"/>
+      <c r="O11" s="47"/>
+      <c r="P11" s="50"/>
+      <c r="Q11" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R11" s="40"/>
+      <c r="S11" s="40"/>
+      <c r="T11" s="40"/>
+      <c r="U11" s="41"/>
+      <c r="W11" s="32"/>
+      <c r="X11" s="33"/>
+      <c r="Y11" s="33"/>
+    </row>
+    <row r="12" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B12" s="159"/>
+      <c r="C12" s="160"/>
+      <c r="D12" s="161"/>
+      <c r="E12" s="136">
+        <v>7</v>
+      </c>
+      <c r="F12" s="145" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="146"/>
+      <c r="H12" s="146"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="47"/>
+      <c r="K12" s="134">
+        <v>1</v>
+      </c>
+      <c r="L12" s="38"/>
+      <c r="M12" s="47"/>
+      <c r="N12" s="47"/>
+      <c r="O12" s="47"/>
+      <c r="P12" s="50"/>
+      <c r="Q12" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R12" s="52"/>
+      <c r="S12" s="40"/>
+      <c r="T12" s="40"/>
+      <c r="U12" s="49"/>
+      <c r="W12" s="32"/>
+      <c r="X12" s="33"/>
+      <c r="Y12" s="33"/>
+    </row>
+    <row r="13" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="162"/>
+      <c r="C13" s="163"/>
+      <c r="D13" s="164"/>
+      <c r="E13" s="136">
+        <v>8</v>
+      </c>
+      <c r="F13" s="145" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="146"/>
+      <c r="H13" s="146"/>
+      <c r="I13" s="46"/>
+      <c r="J13" s="47"/>
+      <c r="K13" s="134">
+        <v>1</v>
+      </c>
+      <c r="L13" s="38"/>
+      <c r="M13" s="47"/>
+      <c r="N13" s="47"/>
+      <c r="O13" s="47"/>
+      <c r="P13" s="50"/>
+      <c r="Q13" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R13" s="52"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="40"/>
+      <c r="U13" s="49"/>
+      <c r="W13" s="32"/>
+      <c r="X13" s="33"/>
+      <c r="Y13" s="33"/>
+    </row>
+    <row r="14" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="156" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="157"/>
+      <c r="D14" s="158"/>
+      <c r="E14" s="135">
+        <v>9</v>
+      </c>
+      <c r="F14" s="145" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="146"/>
+      <c r="H14" s="146"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="134">
+        <v>1</v>
+      </c>
+      <c r="L14" s="134">
+        <v>1</v>
+      </c>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="50"/>
+      <c r="Q14" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R14" s="40"/>
+      <c r="S14" s="40"/>
+      <c r="T14" s="40"/>
+      <c r="U14" s="41"/>
+      <c r="W14" s="32"/>
+      <c r="X14" s="33"/>
+      <c r="Y14" s="33"/>
+    </row>
+    <row r="15" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="159"/>
+      <c r="C15" s="160"/>
+      <c r="D15" s="161"/>
+      <c r="E15" s="136">
+        <v>10</v>
+      </c>
+      <c r="F15" s="145" t="s">
+        <v>35</v>
+      </c>
+      <c r="G15" s="146"/>
+      <c r="H15" s="146"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="47"/>
+      <c r="L15" s="134">
+        <v>3</v>
+      </c>
+      <c r="M15" s="47"/>
+      <c r="N15" s="47"/>
+      <c r="O15" s="47"/>
+      <c r="P15" s="50"/>
+      <c r="Q15" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R15" s="52"/>
+      <c r="S15" s="40"/>
+      <c r="T15" s="40"/>
+      <c r="U15" s="41"/>
+      <c r="W15" s="32"/>
+      <c r="X15" s="33"/>
+      <c r="Y15" s="33"/>
+    </row>
+    <row r="16" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="159"/>
+      <c r="C16" s="160"/>
+      <c r="D16" s="161"/>
+      <c r="E16" s="136">
+        <v>11</v>
+      </c>
+      <c r="F16" s="145" t="s">
+        <v>36</v>
+      </c>
+      <c r="G16" s="146"/>
+      <c r="H16" s="146"/>
+      <c r="I16" s="46"/>
+      <c r="J16" s="47"/>
+      <c r="K16" s="47"/>
+      <c r="L16" s="134">
+        <v>1</v>
+      </c>
+      <c r="M16" s="47"/>
+      <c r="N16" s="47"/>
+      <c r="O16" s="47"/>
+      <c r="P16" s="50"/>
+      <c r="Q16" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R16" s="40"/>
+      <c r="S16" s="40"/>
+      <c r="T16" s="40"/>
+      <c r="U16" s="41"/>
+      <c r="W16" s="32"/>
+      <c r="X16" s="33"/>
+      <c r="Y16" s="33"/>
+    </row>
+    <row r="17" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B17" s="159"/>
+      <c r="C17" s="160"/>
+      <c r="D17" s="161"/>
+      <c r="E17" s="135">
+        <v>12</v>
+      </c>
+      <c r="F17" s="145" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" s="146"/>
+      <c r="H17" s="146"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="47"/>
+      <c r="K17" s="47"/>
+      <c r="M17" s="134">
+        <v>2</v>
+      </c>
+      <c r="N17" s="47"/>
+      <c r="O17" s="47"/>
+      <c r="P17" s="50"/>
+      <c r="Q17" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R17" s="52"/>
+      <c r="S17" s="40"/>
+      <c r="T17" s="40"/>
+      <c r="U17" s="49"/>
+      <c r="W17" s="32"/>
+      <c r="X17" s="33"/>
+      <c r="Y17" s="33"/>
+    </row>
+    <row r="18" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="159"/>
+      <c r="C18" s="160"/>
+      <c r="D18" s="161"/>
+      <c r="E18" s="136">
+        <v>13</v>
+      </c>
+      <c r="F18" s="145" t="s">
+        <v>38</v>
+      </c>
+      <c r="G18" s="146"/>
+      <c r="H18" s="146"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="47"/>
+      <c r="K18" s="47"/>
+      <c r="L18" s="47"/>
+      <c r="M18" s="134">
+        <v>3</v>
+      </c>
+      <c r="N18" s="47"/>
+      <c r="O18" s="47"/>
+      <c r="P18" s="50"/>
+      <c r="Q18" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R18" s="40"/>
+      <c r="S18" s="40"/>
+      <c r="T18" s="40"/>
+      <c r="U18" s="41"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="33"/>
+      <c r="Y18" s="33"/>
+    </row>
+    <row r="19" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="159"/>
+      <c r="C19" s="160"/>
+      <c r="D19" s="161"/>
+      <c r="E19" s="136">
+        <v>14</v>
+      </c>
+      <c r="F19" s="145" t="s">
+        <v>39</v>
+      </c>
+      <c r="G19" s="146"/>
+      <c r="H19" s="146"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="47"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="47"/>
+      <c r="M19" s="47"/>
+      <c r="N19" s="134">
+        <v>1</v>
+      </c>
+      <c r="O19" s="47"/>
+      <c r="P19" s="50"/>
+      <c r="Q19" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R19" s="215"/>
+      <c r="S19" s="52"/>
+      <c r="T19" s="40"/>
+      <c r="U19" s="49"/>
+      <c r="W19" s="32"/>
+      <c r="X19" s="33"/>
+      <c r="Y19" s="33"/>
+    </row>
+    <row r="20" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B20" s="159"/>
+      <c r="C20" s="160"/>
+      <c r="D20" s="161"/>
+      <c r="E20" s="135">
+        <v>15</v>
+      </c>
+      <c r="F20" s="145" t="s">
+        <v>40</v>
+      </c>
+      <c r="G20" s="146"/>
+      <c r="H20" s="146"/>
+      <c r="I20" s="46"/>
+      <c r="J20" s="47"/>
+      <c r="K20" s="47"/>
+      <c r="L20" s="47"/>
+      <c r="M20" s="47"/>
+      <c r="N20" s="134">
+        <v>2</v>
+      </c>
+      <c r="O20" s="47"/>
+      <c r="P20" s="50"/>
+      <c r="Q20" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R20" s="40"/>
+      <c r="S20" s="40"/>
+      <c r="T20" s="40"/>
+      <c r="U20" s="41"/>
+      <c r="W20" s="32"/>
+      <c r="X20" s="33"/>
+      <c r="Y20" s="33"/>
+    </row>
+    <row r="21" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B21" s="159"/>
+      <c r="C21" s="160"/>
+      <c r="D21" s="161"/>
+      <c r="E21" s="136">
+        <v>16</v>
+      </c>
+      <c r="F21" s="145" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="159"/>
-      <c r="H7" s="159"/>
-      <c r="I7" s="150">
+      <c r="G21" s="146"/>
+      <c r="H21" s="146"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="47"/>
+      <c r="K21" s="47"/>
+      <c r="L21" s="47"/>
+      <c r="M21" s="47"/>
+      <c r="N21" s="134">
         <v>2</v>
       </c>
-      <c r="J7" s="42"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="42"/>
-      <c r="M7" s="42"/>
-      <c r="N7" s="42"/>
-      <c r="O7" s="42"/>
-      <c r="P7" s="42"/>
-      <c r="Q7" s="42"/>
-      <c r="R7" s="42"/>
-      <c r="S7" s="43"/>
-      <c r="T7" s="31"/>
-      <c r="U7" s="44"/>
-      <c r="V7" s="44"/>
-      <c r="W7" s="45"/>
-      <c r="Y7" s="36"/>
-      <c r="Z7" s="37"/>
-      <c r="AA7" s="37"/>
+      <c r="O21" s="134">
+        <v>1</v>
+      </c>
+      <c r="P21" s="50"/>
+      <c r="Q21" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R21" s="40"/>
+      <c r="S21" s="52"/>
+      <c r="T21" s="40"/>
+      <c r="U21" s="49"/>
+      <c r="W21" s="32"/>
+      <c r="X21" s="33"/>
+      <c r="Y21" s="33"/>
     </row>
-    <row r="8" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B8" s="163"/>
-      <c r="C8" s="164"/>
-      <c r="D8" s="165"/>
-      <c r="E8" s="155">
+    <row r="22" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="159"/>
+      <c r="C22" s="160"/>
+      <c r="D22" s="161"/>
+      <c r="E22" s="136">
+        <v>17</v>
+      </c>
+      <c r="F22" s="145" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" s="146"/>
+      <c r="H22" s="146"/>
+      <c r="I22" s="46"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="47"/>
+      <c r="M22" s="47"/>
+      <c r="N22" s="47"/>
+      <c r="O22" s="134">
+        <v>2</v>
+      </c>
+      <c r="P22" s="50"/>
+      <c r="Q22" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R22" s="40"/>
+      <c r="S22" s="40"/>
+      <c r="T22" s="40"/>
+      <c r="U22" s="41"/>
+      <c r="W22" s="32"/>
+      <c r="X22" s="33"/>
+      <c r="Y22" s="33"/>
+    </row>
+    <row r="23" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="162"/>
+      <c r="C23" s="163"/>
+      <c r="D23" s="164"/>
+      <c r="E23" s="135">
+        <v>18</v>
+      </c>
+      <c r="F23" s="145" t="s">
+        <v>42</v>
+      </c>
+      <c r="G23" s="146"/>
+      <c r="H23" s="146"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="47"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="47"/>
+      <c r="M23" s="47"/>
+      <c r="N23" s="47"/>
+      <c r="O23" s="134">
+        <v>2</v>
+      </c>
+      <c r="P23" s="204">
+        <v>1</v>
+      </c>
+      <c r="Q23" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R23" s="40"/>
+      <c r="S23" s="52"/>
+      <c r="T23" s="40"/>
+      <c r="U23" s="49"/>
+      <c r="W23" s="32"/>
+      <c r="X23" s="33"/>
+      <c r="Y23" s="33"/>
+    </row>
+    <row r="24" spans="2:25" s="31" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B24" s="156" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="157"/>
+      <c r="D24" s="158"/>
+      <c r="E24" s="135">
+        <v>19</v>
+      </c>
+      <c r="F24" s="145" t="s">
+        <v>44</v>
+      </c>
+      <c r="G24" s="146"/>
+      <c r="H24" s="146"/>
+      <c r="I24" s="46"/>
+      <c r="J24" s="47"/>
+      <c r="K24" s="47"/>
+      <c r="L24" s="47"/>
+      <c r="M24" s="47"/>
+      <c r="N24" s="47"/>
+      <c r="O24" s="47"/>
+      <c r="P24" s="204">
+        <v>2</v>
+      </c>
+      <c r="Q24" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R24" s="40"/>
+      <c r="S24" s="40"/>
+      <c r="T24" s="40"/>
+      <c r="U24" s="41"/>
+      <c r="W24" s="32"/>
+      <c r="X24" s="33"/>
+      <c r="Y24" s="33"/>
+    </row>
+    <row r="25" spans="2:25" s="31" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="162"/>
+      <c r="C25" s="163"/>
+      <c r="D25" s="164"/>
+      <c r="E25" s="136">
+        <v>20</v>
+      </c>
+      <c r="F25" s="145" t="s">
+        <v>45</v>
+      </c>
+      <c r="G25" s="146"/>
+      <c r="H25" s="146"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="47"/>
+      <c r="K25" s="47"/>
+      <c r="L25" s="47"/>
+      <c r="M25" s="47"/>
+      <c r="N25" s="47"/>
+      <c r="O25" s="47"/>
+      <c r="P25" s="204">
+        <v>2</v>
+      </c>
+      <c r="Q25" s="214" t="s">
+        <v>11</v>
+      </c>
+      <c r="R25" s="40"/>
+      <c r="S25" s="215"/>
+      <c r="T25" s="52"/>
+      <c r="U25" s="49"/>
+      <c r="W25" s="32"/>
+      <c r="X25" s="33"/>
+      <c r="Y25" s="33"/>
+    </row>
+    <row r="26" spans="2:25" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="65"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="135"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="46"/>
+      <c r="J26" s="47"/>
+      <c r="K26" s="47"/>
+      <c r="L26" s="47"/>
+      <c r="M26" s="53"/>
+      <c r="N26" s="47"/>
+      <c r="O26" s="47"/>
+      <c r="P26" s="50"/>
+      <c r="Q26" s="216"/>
+      <c r="R26" s="40"/>
+      <c r="S26" s="40"/>
+      <c r="T26" s="40"/>
+      <c r="U26" s="41"/>
+      <c r="W26" s="32"/>
+      <c r="X26" s="33"/>
+      <c r="Y26" s="33"/>
+    </row>
+    <row r="27" spans="2:25" s="31" customFormat="1" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="54"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="56"/>
+      <c r="E27" s="57"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="140"/>
+      <c r="J27" s="141"/>
+      <c r="K27" s="141"/>
+      <c r="L27" s="141"/>
+      <c r="M27" s="141"/>
+      <c r="N27" s="141"/>
+      <c r="O27" s="141"/>
+      <c r="P27" s="205"/>
+      <c r="Q27" s="217"/>
+      <c r="R27" s="218"/>
+      <c r="S27" s="218"/>
+      <c r="T27" s="218"/>
+      <c r="U27" s="219"/>
+      <c r="W27" s="32"/>
+      <c r="X27" s="33"/>
+      <c r="Y27" s="33"/>
+    </row>
+    <row r="28" spans="2:25" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="59"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="61"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="63" t="s">
+        <v>4</v>
+      </c>
+      <c r="G28" s="64"/>
+      <c r="H28" s="64"/>
+      <c r="I28" s="137"/>
+      <c r="J28" s="138"/>
+      <c r="K28" s="138"/>
+      <c r="L28" s="138"/>
+      <c r="M28" s="139" t="s">
+        <v>25</v>
+      </c>
+      <c r="N28" s="138"/>
+      <c r="O28" s="139"/>
+      <c r="P28" s="138"/>
+      <c r="Q28" s="206"/>
+      <c r="R28" s="139"/>
+      <c r="S28" s="139"/>
+      <c r="T28" s="207"/>
+      <c r="U28" s="208"/>
+      <c r="W28" s="32"/>
+      <c r="X28" s="33"/>
+      <c r="Y28" s="33"/>
+    </row>
+    <row r="29" spans="2:25" s="31" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="65"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="35"/>
+      <c r="E29" s="36">
+        <v>1</v>
+      </c>
+      <c r="F29" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="I29" s="37"/>
+      <c r="J29" s="131"/>
+      <c r="K29" s="38"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="38"/>
+      <c r="N29" s="38"/>
+      <c r="O29" s="38"/>
+      <c r="P29" s="38"/>
+      <c r="Q29" s="66"/>
+      <c r="R29" s="40"/>
+      <c r="S29" s="52"/>
+      <c r="T29" s="40"/>
+      <c r="U29" s="67"/>
+      <c r="W29" s="32"/>
+      <c r="X29" s="33"/>
+      <c r="Y29" s="33"/>
+    </row>
+    <row r="30" spans="2:25" s="31" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="65"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="36">
+        <v>2</v>
+      </c>
+      <c r="F30" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="I30" s="37"/>
+      <c r="J30" s="130"/>
+      <c r="K30" s="38"/>
+      <c r="L30" s="38"/>
+      <c r="M30" s="38"/>
+      <c r="N30" s="38"/>
+      <c r="O30" s="38"/>
+      <c r="P30" s="38"/>
+      <c r="Q30" s="69"/>
+      <c r="R30" s="40"/>
+      <c r="S30" s="52"/>
+      <c r="T30" s="70"/>
+      <c r="U30" s="67"/>
+      <c r="W30" s="32"/>
+      <c r="X30" s="33"/>
+      <c r="Y30" s="33"/>
+    </row>
+    <row r="31" spans="2:25" s="31" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="27"/>
+      <c r="C31" s="42"/>
+      <c r="D31" s="43"/>
+      <c r="E31" s="44">
         <v>3</v>
       </c>
-      <c r="F8" s="158" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="159"/>
-      <c r="H8" s="159"/>
-      <c r="I8" s="151">
-        <v>1</v>
-      </c>
-      <c r="J8" s="152">
-        <v>1</v>
-      </c>
-      <c r="K8" s="51"/>
-      <c r="L8" s="42"/>
-      <c r="M8" s="51"/>
-      <c r="N8" s="51"/>
-      <c r="O8" s="51"/>
-      <c r="P8" s="51"/>
-      <c r="Q8" s="51"/>
-      <c r="R8" s="51"/>
-      <c r="S8" s="52"/>
-      <c r="U8" s="44"/>
-      <c r="V8" s="44"/>
-      <c r="W8" s="53"/>
-      <c r="Y8" s="36"/>
-      <c r="Z8" s="37"/>
-      <c r="AA8" s="37"/>
+      <c r="F31" s="142" t="s">
+        <v>65</v>
+      </c>
+      <c r="G31" s="143"/>
+      <c r="H31" s="144"/>
+      <c r="I31" s="46"/>
+      <c r="J31" s="130"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="47"/>
+      <c r="M31" s="47"/>
+      <c r="N31" s="47"/>
+      <c r="O31" s="47"/>
+      <c r="P31" s="47"/>
+      <c r="Q31" s="39"/>
+      <c r="R31" s="71"/>
+      <c r="S31" s="40"/>
+      <c r="T31" s="52"/>
+      <c r="U31" s="72"/>
+      <c r="W31" s="32"/>
+      <c r="X31" s="33"/>
+      <c r="Y31" s="33"/>
     </row>
-    <row r="9" spans="2:27" s="35" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="166"/>
-      <c r="C9" s="167"/>
-      <c r="D9" s="168"/>
-      <c r="E9" s="155">
+    <row r="32" spans="2:25" s="31" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="27"/>
+      <c r="C32" s="42"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="44">
         <v>4</v>
       </c>
-      <c r="F9" s="158" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="159"/>
-      <c r="H9" s="159"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="152">
-        <v>2</v>
-      </c>
-      <c r="K9" s="54"/>
-      <c r="L9" s="42"/>
-      <c r="M9" s="55"/>
-      <c r="N9" s="51"/>
-      <c r="O9" s="51"/>
-      <c r="P9" s="51"/>
-      <c r="Q9" s="51"/>
-      <c r="R9" s="51"/>
-      <c r="S9" s="43"/>
-      <c r="T9" s="44"/>
-      <c r="U9" s="44"/>
-      <c r="V9" s="44"/>
-      <c r="W9" s="45"/>
-      <c r="Y9" s="36"/>
-      <c r="Z9" s="37"/>
-      <c r="AA9" s="37"/>
+      <c r="F32" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="I32" s="46"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="47"/>
+      <c r="L32" s="47"/>
+      <c r="M32" s="47"/>
+      <c r="N32" s="47"/>
+      <c r="O32" s="47"/>
+      <c r="P32" s="47"/>
+      <c r="Q32" s="39"/>
+      <c r="R32" s="52"/>
+      <c r="S32" s="40"/>
+      <c r="T32" s="73"/>
+      <c r="U32" s="41"/>
+      <c r="W32" s="32"/>
+      <c r="X32" s="33"/>
+      <c r="Y32" s="33"/>
     </row>
-    <row r="10" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B10" s="169" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" s="170"/>
-      <c r="D10" s="171"/>
-      <c r="E10" s="48">
+    <row r="33" spans="2:25" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="27"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="43"/>
+      <c r="E33" s="44">
         <v>5</v>
       </c>
-      <c r="F10" s="158" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="159"/>
-      <c r="H10" s="159"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="152">
-        <v>2</v>
-      </c>
-      <c r="K10" s="54"/>
-      <c r="L10" s="42"/>
-      <c r="M10" s="55"/>
-      <c r="N10" s="51"/>
-      <c r="O10" s="51"/>
-      <c r="P10" s="51"/>
-      <c r="Q10" s="51"/>
-      <c r="R10" s="51"/>
-      <c r="S10" s="52"/>
-      <c r="T10" s="44"/>
-      <c r="V10" s="44"/>
-      <c r="W10" s="53"/>
-      <c r="Y10" s="36"/>
-      <c r="Z10" s="37"/>
-      <c r="AA10" s="37"/>
+      <c r="I33" s="46"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="47"/>
+      <c r="L33" s="47"/>
+      <c r="M33" s="47"/>
+      <c r="N33" s="47"/>
+      <c r="O33" s="47"/>
+      <c r="P33" s="47"/>
+      <c r="Q33" s="48"/>
+      <c r="R33" s="40"/>
+      <c r="S33" s="40"/>
+      <c r="T33" s="40"/>
+      <c r="U33" s="49"/>
+      <c r="W33" s="32"/>
+      <c r="X33" s="33"/>
+      <c r="Y33" s="33"/>
     </row>
-    <row r="11" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B11" s="172"/>
-      <c r="C11" s="173"/>
-      <c r="D11" s="174"/>
-      <c r="E11" s="48">
+    <row r="34" spans="2:25" s="31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="74"/>
+      <c r="C34" s="75"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="78"/>
+      <c r="G34" s="79"/>
+      <c r="H34" s="79"/>
+      <c r="I34" s="80"/>
+      <c r="J34" s="81"/>
+      <c r="K34" s="81"/>
+      <c r="L34" s="81"/>
+      <c r="M34" s="81"/>
+      <c r="N34" s="81"/>
+      <c r="O34" s="81"/>
+      <c r="P34" s="81"/>
+      <c r="Q34" s="80"/>
+      <c r="R34" s="81"/>
+      <c r="S34" s="81"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
+      <c r="W34" s="32"/>
+      <c r="X34" s="33"/>
+      <c r="Y34" s="33"/>
+    </row>
+    <row r="35" spans="2:25" s="31" customFormat="1" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="84"/>
+      <c r="C35" s="85"/>
+      <c r="D35" s="86"/>
+      <c r="E35" s="87"/>
+      <c r="F35" s="88"/>
+      <c r="G35" s="89"/>
+      <c r="H35" s="90" t="s">
+        <v>5</v>
+      </c>
+      <c r="I35" s="91"/>
+      <c r="J35" s="92"/>
+      <c r="K35" s="92"/>
+      <c r="L35" s="92"/>
+      <c r="M35" s="92"/>
+      <c r="N35" s="92"/>
+      <c r="O35" s="92"/>
+      <c r="P35" s="92"/>
+      <c r="Q35" s="91"/>
+      <c r="R35" s="92"/>
+      <c r="S35" s="92"/>
+      <c r="T35" s="93"/>
+      <c r="U35" s="94"/>
+      <c r="W35" s="32"/>
+      <c r="X35" s="33"/>
+      <c r="Y35" s="33"/>
+    </row>
+    <row r="36" spans="2:25" s="31" customFormat="1" ht="4.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="95"/>
+      <c r="C36" s="96"/>
+      <c r="D36" s="97"/>
+      <c r="E36" s="98"/>
+      <c r="F36" s="99"/>
+      <c r="G36" s="99"/>
+      <c r="H36" s="99"/>
+      <c r="I36" s="100"/>
+      <c r="J36" s="101"/>
+      <c r="K36" s="101"/>
+      <c r="L36" s="101"/>
+      <c r="M36" s="101"/>
+      <c r="N36" s="101"/>
+      <c r="O36" s="101"/>
+      <c r="P36" s="101"/>
+      <c r="Q36" s="100"/>
+      <c r="R36" s="101"/>
+      <c r="S36" s="101"/>
+      <c r="T36" s="102"/>
+      <c r="U36" s="103"/>
+      <c r="V36" s="1"/>
+      <c r="W36" s="32"/>
+      <c r="X36" s="33"/>
+      <c r="Y36" s="33"/>
+    </row>
+    <row r="37" spans="2:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="178"/>
+      <c r="C37" s="178"/>
+      <c r="D37" s="181"/>
+      <c r="F37" s="104"/>
+      <c r="G37" s="105"/>
+      <c r="H37" s="105"/>
+      <c r="I37" s="183" t="s">
+        <v>51</v>
+      </c>
+      <c r="J37" s="183" t="s">
+        <v>52</v>
+      </c>
+      <c r="K37" s="183" t="s">
+        <v>53</v>
+      </c>
+      <c r="L37" s="183" t="s">
+        <v>54</v>
+      </c>
+      <c r="M37" s="183" t="s">
+        <v>55</v>
+      </c>
+      <c r="N37" s="183" t="s">
+        <v>56</v>
+      </c>
+      <c r="O37" s="183" t="s">
+        <v>57</v>
+      </c>
+      <c r="P37" s="183" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q37" s="187" t="s">
+        <v>14</v>
+      </c>
+      <c r="R37" s="190" t="s">
+        <v>15</v>
+      </c>
+      <c r="S37" s="190" t="s">
+        <v>16</v>
+      </c>
+      <c r="T37" s="190" t="s">
+        <v>18</v>
+      </c>
+      <c r="U37" s="198" t="s">
+        <v>17</v>
+      </c>
+      <c r="W37" s="32"/>
+      <c r="X37" s="33"/>
+      <c r="Y37" s="33"/>
+    </row>
+    <row r="38" spans="2:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="179"/>
+      <c r="C38" s="179"/>
+      <c r="D38" s="181"/>
+      <c r="F38" s="106"/>
+      <c r="G38" s="105"/>
+      <c r="H38" s="105"/>
+      <c r="I38" s="183"/>
+      <c r="J38" s="183"/>
+      <c r="K38" s="183"/>
+      <c r="L38" s="183"/>
+      <c r="M38" s="183"/>
+      <c r="N38" s="183"/>
+      <c r="O38" s="183"/>
+      <c r="P38" s="183"/>
+      <c r="Q38" s="188"/>
+      <c r="R38" s="191"/>
+      <c r="S38" s="191"/>
+      <c r="T38" s="190"/>
+      <c r="U38" s="199"/>
+      <c r="W38" s="32"/>
+      <c r="X38" s="33"/>
+      <c r="Y38" s="33"/>
+    </row>
+    <row r="39" spans="2:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="179"/>
+      <c r="C39" s="179"/>
+      <c r="D39" s="181"/>
+      <c r="F39" s="104"/>
+      <c r="G39" s="105"/>
+      <c r="H39" s="105"/>
+      <c r="I39" s="183"/>
+      <c r="J39" s="183"/>
+      <c r="K39" s="183"/>
+      <c r="L39" s="183"/>
+      <c r="M39" s="183"/>
+      <c r="N39" s="183"/>
+      <c r="O39" s="183"/>
+      <c r="P39" s="183"/>
+      <c r="Q39" s="188"/>
+      <c r="R39" s="191"/>
+      <c r="S39" s="191"/>
+      <c r="T39" s="190"/>
+      <c r="U39" s="199"/>
+      <c r="X39" s="33"/>
+      <c r="Y39" s="33"/>
+    </row>
+    <row r="40" spans="2:25" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="179"/>
+      <c r="C40" s="179"/>
+      <c r="D40" s="181"/>
+      <c r="F40" s="107"/>
+      <c r="G40" s="105"/>
+      <c r="H40" s="105"/>
+      <c r="I40" s="184"/>
+      <c r="J40" s="184"/>
+      <c r="K40" s="184"/>
+      <c r="L40" s="184"/>
+      <c r="M40" s="184"/>
+      <c r="N40" s="184"/>
+      <c r="O40" s="184"/>
+      <c r="P40" s="184"/>
+      <c r="Q40" s="189"/>
+      <c r="R40" s="192"/>
+      <c r="S40" s="192"/>
+      <c r="T40" s="197"/>
+      <c r="U40" s="200"/>
+      <c r="X40" s="2"/>
+      <c r="Y40" s="2"/>
+    </row>
+    <row r="41" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="179"/>
+      <c r="C41" s="179"/>
+      <c r="D41" s="181"/>
+      <c r="F41" s="107"/>
+      <c r="G41" s="107"/>
+      <c r="H41" s="107"/>
+      <c r="I41" s="108"/>
+      <c r="J41" s="109"/>
+      <c r="K41" s="109"/>
+      <c r="L41" s="109"/>
+      <c r="M41" s="109"/>
+      <c r="N41" s="109"/>
+      <c r="O41" s="109"/>
+      <c r="P41" s="109"/>
+      <c r="Q41" s="109"/>
+      <c r="R41" s="109"/>
+      <c r="S41" s="109"/>
+      <c r="T41" s="109"/>
+      <c r="U41" s="110"/>
+      <c r="X41" s="33"/>
+      <c r="Y41" s="33"/>
+    </row>
+    <row r="42" spans="2:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="179"/>
+      <c r="C42" s="179"/>
+      <c r="D42" s="181"/>
+      <c r="E42" s="111"/>
+      <c r="F42" s="107"/>
+      <c r="G42" s="106"/>
+      <c r="H42" s="106"/>
+      <c r="I42" s="112"/>
+      <c r="J42" s="113"/>
+      <c r="K42" s="113"/>
+      <c r="L42" s="113"/>
+      <c r="M42" s="113"/>
+      <c r="N42" s="113"/>
+      <c r="O42" s="113"/>
+      <c r="P42" s="113"/>
+      <c r="Q42" s="113"/>
+      <c r="R42" s="113"/>
+      <c r="S42" s="113"/>
+      <c r="T42" s="113"/>
+      <c r="U42" s="114"/>
+      <c r="X42" s="2"/>
+      <c r="Y42" s="2"/>
+    </row>
+    <row r="43" spans="2:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="179"/>
+      <c r="C43" s="179"/>
+      <c r="D43" s="181"/>
+      <c r="F43" s="104"/>
+      <c r="G43" s="106"/>
+      <c r="H43" s="106"/>
+      <c r="I43" s="112"/>
+      <c r="J43" s="113"/>
+      <c r="K43" s="113"/>
+      <c r="L43" s="113"/>
+      <c r="M43" s="113"/>
+      <c r="N43" s="113"/>
+      <c r="O43" s="113"/>
+      <c r="P43" s="113"/>
+      <c r="Q43" s="113"/>
+      <c r="R43" s="113"/>
+      <c r="S43" s="113"/>
+      <c r="T43" s="113"/>
+      <c r="U43" s="114"/>
+      <c r="X43" s="33"/>
+      <c r="Y43" s="33"/>
+    </row>
+    <row r="44" spans="2:25" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B44" s="179"/>
+      <c r="C44" s="179"/>
+      <c r="D44" s="181"/>
+      <c r="F44" s="104"/>
+      <c r="G44" s="106"/>
+      <c r="H44" s="115"/>
+      <c r="I44" s="112"/>
+      <c r="J44" s="113"/>
+      <c r="K44" s="113"/>
+      <c r="L44" s="113"/>
+      <c r="M44" s="113"/>
+      <c r="N44" s="113"/>
+      <c r="O44" s="113"/>
+      <c r="P44" s="113"/>
+      <c r="Q44" s="113"/>
+      <c r="R44" s="113"/>
+      <c r="S44" s="113"/>
+      <c r="T44" s="113"/>
+      <c r="U44" s="114"/>
+      <c r="X44" s="2"/>
+      <c r="Y44" s="2"/>
+    </row>
+    <row r="45" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="179"/>
+      <c r="C45" s="179"/>
+      <c r="D45" s="181"/>
+      <c r="F45" s="104"/>
+      <c r="G45" s="104"/>
+      <c r="H45" s="104"/>
+      <c r="I45" s="112"/>
+      <c r="J45" s="113"/>
+      <c r="K45" s="113"/>
+      <c r="L45" s="113"/>
+      <c r="M45" s="113"/>
+      <c r="N45" s="113"/>
+      <c r="O45" s="113"/>
+      <c r="P45" s="113"/>
+      <c r="Q45" s="113"/>
+      <c r="R45" s="113"/>
+      <c r="S45" s="113"/>
+      <c r="T45" s="113"/>
+      <c r="U45" s="114"/>
+      <c r="X45" s="33"/>
+      <c r="Y45" s="33"/>
+    </row>
+    <row r="46" spans="2:25" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B46" s="179"/>
+      <c r="C46" s="179"/>
+      <c r="D46" s="181"/>
+      <c r="F46" s="116"/>
+      <c r="I46" s="112"/>
+      <c r="J46" s="113"/>
+      <c r="K46" s="113"/>
+      <c r="L46" s="113"/>
+      <c r="M46" s="113"/>
+      <c r="N46" s="113"/>
+      <c r="O46" s="113"/>
+      <c r="P46" s="113"/>
+      <c r="Q46" s="113"/>
+      <c r="R46" s="113"/>
+      <c r="S46" s="113"/>
+      <c r="T46" s="113"/>
+      <c r="U46" s="114"/>
+      <c r="X46" s="2"/>
+      <c r="Y46" s="2"/>
+    </row>
+    <row r="47" spans="2:25" ht="50.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="179"/>
+      <c r="C47" s="179"/>
+      <c r="D47" s="181"/>
+      <c r="E47" s="118"/>
+      <c r="F47" s="118"/>
+      <c r="G47" s="118"/>
+      <c r="H47" s="118"/>
+      <c r="I47" s="119"/>
+      <c r="J47" s="120"/>
+      <c r="K47" s="120"/>
+      <c r="L47" s="120"/>
+      <c r="M47" s="120"/>
+      <c r="N47" s="120"/>
+      <c r="O47" s="120"/>
+      <c r="P47" s="120"/>
+      <c r="Q47" s="120"/>
+      <c r="R47" s="120"/>
+      <c r="S47" s="120"/>
+      <c r="T47" s="120"/>
+      <c r="U47" s="121"/>
+      <c r="X47" s="117"/>
+      <c r="Y47" s="117"/>
+    </row>
+    <row r="48" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="179"/>
+      <c r="C48" s="179"/>
+      <c r="D48" s="181"/>
+      <c r="E48" s="201"/>
+      <c r="F48" s="201"/>
+      <c r="G48" s="201"/>
+      <c r="H48" s="201"/>
+      <c r="I48" s="201"/>
+      <c r="J48" s="201"/>
+      <c r="K48" s="201"/>
+      <c r="L48" s="201"/>
+      <c r="M48" s="201"/>
+      <c r="N48" s="201"/>
+      <c r="O48" s="201"/>
+      <c r="P48" s="201"/>
+      <c r="Q48" s="201"/>
+      <c r="R48" s="201"/>
+      <c r="S48" s="201"/>
+      <c r="T48" s="201"/>
+      <c r="U48" s="202"/>
+    </row>
+    <row r="49" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="179"/>
+      <c r="C49" s="179"/>
+      <c r="D49" s="181"/>
+      <c r="E49" s="195"/>
+      <c r="F49" s="195"/>
+      <c r="G49" s="195"/>
+      <c r="H49" s="195"/>
+      <c r="I49" s="195"/>
+      <c r="J49" s="195"/>
+      <c r="K49" s="195"/>
+      <c r="L49" s="195"/>
+      <c r="M49" s="195"/>
+      <c r="N49" s="195"/>
+      <c r="O49" s="195"/>
+      <c r="P49" s="195"/>
+      <c r="Q49" s="195"/>
+      <c r="R49" s="195"/>
+      <c r="S49" s="195"/>
+      <c r="T49" s="195"/>
+      <c r="U49" s="196"/>
+    </row>
+    <row r="50" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="179"/>
+      <c r="C50" s="179"/>
+      <c r="D50" s="181"/>
+      <c r="E50" s="195"/>
+      <c r="F50" s="195"/>
+      <c r="G50" s="195"/>
+      <c r="H50" s="195"/>
+      <c r="I50" s="195"/>
+      <c r="J50" s="195"/>
+      <c r="K50" s="195"/>
+      <c r="L50" s="195"/>
+      <c r="M50" s="195"/>
+      <c r="N50" s="195"/>
+      <c r="O50" s="195"/>
+      <c r="P50" s="195"/>
+      <c r="Q50" s="195"/>
+      <c r="R50" s="195"/>
+      <c r="S50" s="195"/>
+      <c r="T50" s="195"/>
+      <c r="U50" s="196"/>
+    </row>
+    <row r="51" spans="2:25" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="180"/>
+      <c r="C51" s="180"/>
+      <c r="D51" s="182"/>
+      <c r="E51" s="185"/>
+      <c r="F51" s="185"/>
+      <c r="G51" s="185"/>
+      <c r="H51" s="185"/>
+      <c r="I51" s="185"/>
+      <c r="J51" s="185"/>
+      <c r="K51" s="185"/>
+      <c r="L51" s="185"/>
+      <c r="M51" s="185"/>
+      <c r="N51" s="185"/>
+      <c r="O51" s="185"/>
+      <c r="P51" s="185"/>
+      <c r="Q51" s="185"/>
+      <c r="R51" s="185"/>
+      <c r="S51" s="185"/>
+      <c r="T51" s="185"/>
+      <c r="U51" s="186"/>
+    </row>
+    <row r="53" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="K53" s="122" t="s">
+        <v>7</v>
+      </c>
+      <c r="L53" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="158" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="159"/>
-      <c r="H11" s="159"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="51"/>
-      <c r="K11" s="152">
-        <v>2</v>
-      </c>
-      <c r="L11" s="42"/>
-      <c r="M11" s="42"/>
-      <c r="N11" s="51"/>
-      <c r="O11" s="51"/>
-      <c r="P11" s="51"/>
-      <c r="Q11" s="51"/>
-      <c r="R11" s="51"/>
-      <c r="S11" s="43"/>
-      <c r="T11" s="44"/>
-      <c r="U11" s="44"/>
-      <c r="V11" s="44"/>
-      <c r="W11" s="45"/>
-      <c r="Y11" s="36"/>
-      <c r="Z11" s="37"/>
-      <c r="AA11" s="37"/>
+      <c r="M53" s="122" t="s">
+        <v>9</v>
+      </c>
+      <c r="N53" s="122" t="s">
+        <v>8</v>
+      </c>
+      <c r="O53" s="123"/>
+      <c r="P53" s="123"/>
+      <c r="Q53" s="124" t="s">
+        <v>11</v>
+      </c>
+      <c r="R53" s="193" t="s">
+        <v>19</v>
+      </c>
+      <c r="S53" s="194"/>
+      <c r="T53" s="123"/>
+      <c r="U53" s="123"/>
+      <c r="V53" s="123"/>
+      <c r="W53" s="123"/>
+      <c r="X53" s="123"/>
+      <c r="Y53" s="123"/>
     </row>
-    <row r="12" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B12" s="172"/>
-      <c r="C12" s="173"/>
-      <c r="D12" s="174"/>
-      <c r="E12" s="48">
+    <row r="54" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="J54" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K54" s="125" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="158" t="s">
-        <v>46</v>
-      </c>
-      <c r="G12" s="159"/>
-      <c r="H12" s="159"/>
-      <c r="I12" s="50"/>
-      <c r="J12" s="51"/>
-      <c r="K12" s="152">
-        <v>1</v>
-      </c>
-      <c r="L12" s="42"/>
-      <c r="M12" s="51"/>
-      <c r="N12" s="51"/>
-      <c r="O12" s="51"/>
-      <c r="P12" s="51"/>
-      <c r="Q12" s="51"/>
-      <c r="R12" s="51"/>
-      <c r="S12" s="43"/>
-      <c r="T12" s="56"/>
-      <c r="U12" s="44"/>
-      <c r="V12" s="44"/>
-      <c r="W12" s="53"/>
-      <c r="Y12" s="36"/>
-      <c r="Z12" s="37"/>
-      <c r="AA12" s="37"/>
+      <c r="L54" s="125" t="s">
+        <v>6</v>
+      </c>
+      <c r="M54" s="125" t="s">
+        <v>9</v>
+      </c>
+      <c r="N54" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="O54" s="53"/>
+      <c r="P54" s="53"/>
+      <c r="Q54" s="126" t="s">
+        <v>12</v>
+      </c>
+      <c r="R54" s="193" t="s">
+        <v>20</v>
+      </c>
+      <c r="S54" s="194"/>
+      <c r="T54" s="53"/>
+      <c r="U54" s="53"/>
+      <c r="V54" s="53"/>
+      <c r="W54" s="53"/>
+      <c r="X54" s="53"/>
+      <c r="Y54" s="53"/>
     </row>
-    <row r="13" spans="2:27" s="35" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="175"/>
-      <c r="C13" s="176"/>
-      <c r="D13" s="177"/>
-      <c r="E13" s="48">
-        <v>7</v>
-      </c>
-      <c r="F13" s="158" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13" s="159"/>
-      <c r="H13" s="159"/>
-      <c r="I13" s="50"/>
-      <c r="J13" s="51"/>
-      <c r="K13" s="152">
-        <v>1</v>
-      </c>
-      <c r="L13" s="42"/>
-      <c r="M13" s="51"/>
-      <c r="N13" s="51"/>
-      <c r="O13" s="51"/>
-      <c r="P13" s="51"/>
-      <c r="Q13" s="51"/>
-      <c r="R13" s="51"/>
-      <c r="S13" s="43"/>
-      <c r="T13" s="56"/>
-      <c r="U13" s="44"/>
-      <c r="V13" s="44"/>
-      <c r="W13" s="53"/>
-      <c r="Y13" s="36"/>
-      <c r="Z13" s="37"/>
-      <c r="AA13" s="37"/>
+    <row r="55" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="Q55" s="127" t="s">
+        <v>13</v>
+      </c>
+      <c r="R55" s="193" t="s">
+        <v>21</v>
+      </c>
+      <c r="S55" s="194"/>
+      <c r="W55" s="1"/>
+      <c r="X55" s="1"/>
+      <c r="Y55" s="1"/>
     </row>
-    <row r="14" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B14" s="169" t="s">
-        <v>62</v>
-      </c>
-      <c r="C14" s="170"/>
-      <c r="D14" s="171"/>
-      <c r="E14" s="48">
-        <v>8</v>
-      </c>
-      <c r="F14" s="158" t="s">
-        <v>48</v>
-      </c>
-      <c r="G14" s="159"/>
-      <c r="H14" s="159"/>
-      <c r="I14" s="50"/>
-      <c r="J14" s="51"/>
-      <c r="K14" s="152">
-        <v>1</v>
-      </c>
-      <c r="L14" s="152">
-        <v>1</v>
-      </c>
-      <c r="M14" s="51"/>
-      <c r="N14" s="51"/>
-      <c r="O14" s="51"/>
-      <c r="P14" s="51"/>
-      <c r="Q14" s="51"/>
-      <c r="R14" s="51"/>
-      <c r="S14" s="43"/>
-      <c r="T14" s="44"/>
-      <c r="U14" s="44"/>
-      <c r="V14" s="44"/>
-      <c r="W14" s="45"/>
-      <c r="Y14" s="36"/>
-      <c r="Z14" s="37"/>
-      <c r="AA14" s="37"/>
+    <row r="56" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="W56" s="1"/>
+      <c r="X56" s="1"/>
+      <c r="Y56" s="1"/>
     </row>
-    <row r="15" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B15" s="172"/>
-      <c r="C15" s="173"/>
-      <c r="D15" s="174"/>
-      <c r="E15" s="48">
-        <v>9</v>
-      </c>
-      <c r="F15" s="158" t="s">
-        <v>49</v>
-      </c>
-      <c r="G15" s="159"/>
-      <c r="H15" s="159"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="51"/>
-      <c r="K15" s="51"/>
-      <c r="L15" s="152">
-        <v>3</v>
-      </c>
-      <c r="M15" s="51"/>
-      <c r="N15" s="51"/>
-      <c r="O15" s="51"/>
-      <c r="P15" s="51"/>
-      <c r="Q15" s="51"/>
-      <c r="R15" s="51"/>
-      <c r="S15" s="43"/>
-      <c r="T15" s="56"/>
-      <c r="U15" s="44"/>
-      <c r="V15" s="44"/>
-      <c r="W15" s="45"/>
-      <c r="Y15" s="36"/>
-      <c r="Z15" s="37"/>
-      <c r="AA15" s="37"/>
+    <row r="57" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="K57" s="128"/>
+      <c r="L57" s="129" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="16" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B16" s="172"/>
-      <c r="C16" s="173"/>
-      <c r="D16" s="174"/>
-      <c r="E16" s="48">
-        <v>10</v>
-      </c>
-      <c r="F16" s="158" t="s">
-        <v>50</v>
-      </c>
-      <c r="G16" s="159"/>
-      <c r="H16" s="159"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="51"/>
-      <c r="K16" s="51"/>
-      <c r="L16" s="152">
-        <v>1</v>
-      </c>
-      <c r="M16" s="51"/>
-      <c r="N16" s="51"/>
-      <c r="O16" s="51"/>
-      <c r="P16" s="51"/>
-      <c r="Q16" s="51"/>
-      <c r="R16" s="51"/>
-      <c r="S16" s="43"/>
-      <c r="T16" s="44"/>
-      <c r="U16" s="44"/>
-      <c r="V16" s="44"/>
-      <c r="W16" s="45"/>
-      <c r="Y16" s="36"/>
-      <c r="Z16" s="37"/>
-      <c r="AA16" s="37"/>
+    <row r="58" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="K58" s="130"/>
+      <c r="L58" s="129" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="17" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B17" s="172"/>
-      <c r="C17" s="173"/>
-      <c r="D17" s="174"/>
-      <c r="E17" s="48">
-        <v>11</v>
-      </c>
-      <c r="F17" s="158" t="s">
-        <v>51</v>
-      </c>
-      <c r="G17" s="159"/>
-      <c r="H17" s="159"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="51"/>
-      <c r="K17" s="51"/>
-      <c r="M17" s="152">
-        <v>2</v>
-      </c>
-      <c r="N17" s="51"/>
-      <c r="O17" s="51"/>
-      <c r="P17" s="51"/>
-      <c r="Q17" s="51"/>
-      <c r="R17" s="51"/>
-      <c r="S17" s="43"/>
-      <c r="T17" s="56"/>
-      <c r="U17" s="44"/>
-      <c r="V17" s="44"/>
-      <c r="W17" s="53"/>
-      <c r="Y17" s="36"/>
-      <c r="Z17" s="37"/>
-      <c r="AA17" s="37"/>
-    </row>
-    <row r="18" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B18" s="172"/>
-      <c r="C18" s="173"/>
-      <c r="D18" s="174"/>
-      <c r="E18" s="48">
-        <v>12</v>
-      </c>
-      <c r="F18" s="158" t="s">
-        <v>52</v>
-      </c>
-      <c r="G18" s="159"/>
-      <c r="H18" s="159"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="51"/>
-      <c r="K18" s="51"/>
-      <c r="L18" s="51"/>
-      <c r="M18" s="152">
-        <v>3</v>
-      </c>
-      <c r="N18" s="51"/>
-      <c r="O18" s="51"/>
-      <c r="P18" s="51"/>
-      <c r="Q18" s="51"/>
-      <c r="R18" s="51"/>
-      <c r="S18" s="43"/>
-      <c r="T18" s="44"/>
-      <c r="U18" s="44"/>
-      <c r="V18" s="44"/>
-      <c r="W18" s="45"/>
-      <c r="Y18" s="36"/>
-      <c r="Z18" s="37"/>
-      <c r="AA18" s="37"/>
-    </row>
-    <row r="19" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B19" s="172"/>
-      <c r="C19" s="173"/>
-      <c r="D19" s="174"/>
-      <c r="E19" s="48">
-        <v>13</v>
-      </c>
-      <c r="F19" s="158" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" s="159"/>
-      <c r="H19" s="159"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="51"/>
-      <c r="K19" s="51"/>
-      <c r="L19" s="51"/>
-      <c r="M19" s="51"/>
-      <c r="N19" s="152">
-        <v>1</v>
-      </c>
-      <c r="O19" s="51"/>
-      <c r="P19" s="51"/>
-      <c r="Q19" s="51"/>
-      <c r="R19" s="51"/>
-      <c r="S19" s="43"/>
-      <c r="U19" s="56"/>
-      <c r="V19" s="44"/>
-      <c r="W19" s="53"/>
-      <c r="Y19" s="36"/>
-      <c r="Z19" s="37"/>
-      <c r="AA19" s="37"/>
-    </row>
-    <row r="20" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B20" s="172"/>
-      <c r="C20" s="173"/>
-      <c r="D20" s="174"/>
-      <c r="E20" s="48">
-        <v>14</v>
-      </c>
-      <c r="F20" s="158" t="s">
-        <v>54</v>
-      </c>
-      <c r="G20" s="159"/>
-      <c r="H20" s="159"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="51"/>
-      <c r="K20" s="51"/>
-      <c r="L20" s="51"/>
-      <c r="M20" s="51"/>
-      <c r="N20" s="152">
-        <v>2</v>
-      </c>
-      <c r="O20" s="51"/>
-      <c r="P20" s="51"/>
-      <c r="Q20" s="51"/>
-      <c r="R20" s="51"/>
-      <c r="S20" s="43"/>
-      <c r="T20" s="44"/>
-      <c r="U20" s="44"/>
-      <c r="V20" s="44"/>
-      <c r="W20" s="45"/>
-      <c r="Y20" s="36"/>
-      <c r="Z20" s="37"/>
-      <c r="AA20" s="37"/>
-    </row>
-    <row r="21" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B21" s="172"/>
-      <c r="C21" s="173"/>
-      <c r="D21" s="174"/>
-      <c r="E21" s="48">
-        <v>15</v>
-      </c>
-      <c r="F21" s="158" t="s">
-        <v>55</v>
-      </c>
-      <c r="G21" s="159"/>
-      <c r="H21" s="159"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="51"/>
-      <c r="K21" s="51"/>
-      <c r="L21" s="51"/>
-      <c r="M21" s="51"/>
-      <c r="N21" s="152">
-        <v>2</v>
-      </c>
-      <c r="O21" s="152">
-        <v>1</v>
-      </c>
-      <c r="P21" s="51"/>
-      <c r="Q21" s="51"/>
-      <c r="R21" s="51"/>
-      <c r="S21" s="43"/>
-      <c r="T21" s="44"/>
-      <c r="U21" s="56"/>
-      <c r="V21" s="44"/>
-      <c r="W21" s="53"/>
-      <c r="Y21" s="36"/>
-      <c r="Z21" s="37"/>
-      <c r="AA21" s="37"/>
-    </row>
-    <row r="22" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B22" s="172"/>
-      <c r="C22" s="173"/>
-      <c r="D22" s="174"/>
-      <c r="E22" s="48">
-        <v>16</v>
-      </c>
-      <c r="F22" s="158" t="s">
-        <v>57</v>
-      </c>
-      <c r="G22" s="159"/>
-      <c r="H22" s="159"/>
-      <c r="I22" s="50"/>
-      <c r="J22" s="51"/>
-      <c r="K22" s="51"/>
-      <c r="L22" s="51"/>
-      <c r="M22" s="51"/>
-      <c r="N22" s="51"/>
-      <c r="O22" s="152">
-        <v>2</v>
-      </c>
-      <c r="P22" s="51"/>
-      <c r="Q22" s="51"/>
-      <c r="R22" s="51"/>
-      <c r="S22" s="43"/>
-      <c r="T22" s="44"/>
-      <c r="U22" s="44"/>
-      <c r="V22" s="44"/>
-      <c r="W22" s="45"/>
-      <c r="Y22" s="36"/>
-      <c r="Z22" s="37"/>
-      <c r="AA22" s="37"/>
-    </row>
-    <row r="23" spans="2:27" s="35" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="175"/>
-      <c r="C23" s="176"/>
-      <c r="D23" s="177"/>
-      <c r="E23" s="48">
-        <v>17</v>
-      </c>
-      <c r="F23" s="158" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="159"/>
-      <c r="H23" s="159"/>
-      <c r="I23" s="50"/>
-      <c r="J23" s="51"/>
-      <c r="K23" s="51"/>
-      <c r="L23" s="51"/>
-      <c r="M23" s="51"/>
-      <c r="N23" s="51"/>
-      <c r="O23" s="152">
-        <v>2</v>
-      </c>
-      <c r="P23" s="152">
-        <v>1</v>
-      </c>
-      <c r="Q23" s="51"/>
-      <c r="R23" s="51"/>
-      <c r="S23" s="43"/>
-      <c r="T23" s="44"/>
-      <c r="U23" s="56"/>
-      <c r="V23" s="44"/>
-      <c r="W23" s="53"/>
-      <c r="Y23" s="36"/>
-      <c r="Z23" s="37"/>
-      <c r="AA23" s="37"/>
-    </row>
-    <row r="24" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B24" s="169" t="s">
-        <v>63</v>
-      </c>
-      <c r="C24" s="170"/>
-      <c r="D24" s="171"/>
-      <c r="E24" s="48">
-        <v>18</v>
-      </c>
-      <c r="F24" s="158" t="s">
-        <v>58</v>
-      </c>
-      <c r="G24" s="159"/>
-      <c r="H24" s="159"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="51"/>
-      <c r="K24" s="51"/>
-      <c r="L24" s="51"/>
-      <c r="M24" s="51"/>
-      <c r="N24" s="51"/>
-      <c r="O24" s="51"/>
-      <c r="P24" s="152">
-        <v>2</v>
-      </c>
-      <c r="Q24" s="51"/>
-      <c r="R24" s="51"/>
-      <c r="S24" s="43"/>
-      <c r="T24" s="44"/>
-      <c r="U24" s="44"/>
-      <c r="V24" s="44"/>
-      <c r="W24" s="45"/>
-      <c r="Y24" s="36"/>
-      <c r="Z24" s="37"/>
-      <c r="AA24" s="37"/>
-    </row>
-    <row r="25" spans="2:27" s="35" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="175"/>
-      <c r="C25" s="176"/>
-      <c r="D25" s="177"/>
-      <c r="E25" s="48">
-        <v>19</v>
-      </c>
-      <c r="F25" s="158" t="s">
-        <v>59</v>
-      </c>
-      <c r="G25" s="159"/>
-      <c r="H25" s="159"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="51"/>
-      <c r="L25" s="51"/>
-      <c r="M25" s="51"/>
-      <c r="N25" s="51"/>
-      <c r="O25" s="51"/>
-      <c r="P25" s="152">
-        <v>2</v>
-      </c>
-      <c r="Q25" s="51"/>
-      <c r="R25" s="51"/>
-      <c r="S25" s="43"/>
-      <c r="T25" s="44"/>
-      <c r="V25" s="56"/>
-      <c r="W25" s="53"/>
-      <c r="Y25" s="36"/>
-      <c r="Z25" s="37"/>
-      <c r="AA25" s="37"/>
-    </row>
-    <row r="26" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="82"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="48">
-        <v>20</v>
-      </c>
-      <c r="F26" s="28"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="51"/>
-      <c r="K26" s="51"/>
-      <c r="L26" s="51"/>
-      <c r="M26" s="57"/>
-      <c r="N26" s="51"/>
-      <c r="O26" s="51"/>
-      <c r="P26" s="51"/>
-      <c r="Q26" s="51"/>
-      <c r="R26" s="51"/>
-      <c r="S26" s="43"/>
-      <c r="T26" s="44"/>
-      <c r="U26" s="44"/>
-      <c r="V26" s="44"/>
-      <c r="W26" s="45"/>
-      <c r="Y26" s="36"/>
-      <c r="Z26" s="37"/>
-      <c r="AA26" s="37"/>
-    </row>
-    <row r="27" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="27"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="48">
-        <v>21</v>
-      </c>
-      <c r="F27" s="28"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="58"/>
-      <c r="I27" s="50"/>
-      <c r="J27" s="51"/>
-      <c r="K27" s="51"/>
-      <c r="L27" s="51"/>
-      <c r="M27" s="59"/>
-      <c r="N27" s="51"/>
-      <c r="O27" s="51"/>
-      <c r="P27" s="51"/>
-      <c r="Q27" s="51"/>
-      <c r="R27" s="51"/>
-      <c r="S27" s="43"/>
-      <c r="T27" s="44"/>
-      <c r="V27" s="56"/>
-      <c r="W27" s="53"/>
-      <c r="Y27" s="36"/>
-      <c r="Z27" s="37"/>
-      <c r="AA27" s="37"/>
-    </row>
-    <row r="28" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="27"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="48">
-        <v>22</v>
-      </c>
-      <c r="F28" s="28"/>
-      <c r="G28" s="49"/>
-      <c r="H28" s="58"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="51"/>
-      <c r="K28" s="51"/>
-      <c r="L28" s="51"/>
-      <c r="M28" s="60"/>
-      <c r="N28" s="51"/>
-      <c r="O28" s="51"/>
-      <c r="P28" s="51"/>
-      <c r="Q28" s="51"/>
-      <c r="R28" s="51"/>
-      <c r="S28" s="61"/>
-      <c r="T28" s="44"/>
-      <c r="U28" s="44"/>
-      <c r="V28" s="44"/>
-      <c r="W28" s="45"/>
-      <c r="Y28" s="36"/>
-      <c r="Z28" s="37"/>
-      <c r="AA28" s="37"/>
-    </row>
-    <row r="29" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="27"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="47"/>
-      <c r="E29" s="48">
-        <v>23</v>
-      </c>
-      <c r="F29" s="28"/>
-      <c r="G29" s="58"/>
-      <c r="H29" s="58"/>
-      <c r="I29" s="50"/>
-      <c r="J29" s="51"/>
-      <c r="K29" s="51"/>
-      <c r="L29" s="51"/>
-      <c r="M29" s="51"/>
-      <c r="N29" s="51"/>
-      <c r="O29" s="51"/>
-      <c r="P29" s="51"/>
-      <c r="R29" s="51"/>
-      <c r="S29" s="43"/>
-      <c r="T29" s="44"/>
-      <c r="V29" s="56"/>
-      <c r="W29" s="53"/>
-      <c r="Y29" s="36"/>
-      <c r="Z29" s="37"/>
-      <c r="AA29" s="37"/>
-    </row>
-    <row r="30" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="62"/>
-      <c r="C30" s="63"/>
-      <c r="D30" s="64"/>
-      <c r="E30" s="65">
+    <row r="59" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="K59" s="131"/>
+      <c r="L59" s="129" t="s">
         <v>24</v>
-      </c>
-      <c r="F30" s="28"/>
-      <c r="G30" s="66"/>
-      <c r="H30" s="66"/>
-      <c r="I30" s="67"/>
-      <c r="J30" s="68"/>
-      <c r="K30" s="68"/>
-      <c r="L30" s="68"/>
-      <c r="M30" s="68"/>
-      <c r="N30" s="68"/>
-      <c r="O30" s="68"/>
-      <c r="Q30" s="68"/>
-      <c r="R30" s="68"/>
-      <c r="S30" s="61"/>
-      <c r="T30" s="69"/>
-      <c r="U30" s="69"/>
-      <c r="V30" s="44"/>
-      <c r="W30" s="45"/>
-      <c r="Y30" s="36"/>
-      <c r="Z30" s="37"/>
-      <c r="AA30" s="37"/>
-    </row>
-    <row r="31" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="62"/>
-      <c r="C31" s="63"/>
-      <c r="D31" s="64"/>
-      <c r="E31" s="65">
-        <v>25</v>
-      </c>
-      <c r="F31" s="28"/>
-      <c r="G31" s="66"/>
-      <c r="H31" s="66"/>
-      <c r="I31" s="67"/>
-      <c r="J31" s="68"/>
-      <c r="K31" s="68"/>
-      <c r="L31" s="68"/>
-      <c r="M31" s="68"/>
-      <c r="N31" s="68"/>
-      <c r="O31" s="68"/>
-      <c r="P31" s="68"/>
-      <c r="Q31" s="68"/>
-      <c r="R31" s="68"/>
-      <c r="S31" s="61"/>
-      <c r="T31" s="69"/>
-      <c r="U31" s="69"/>
-      <c r="V31" s="69"/>
-      <c r="W31" s="45"/>
-      <c r="Y31" s="36"/>
-      <c r="Z31" s="37"/>
-      <c r="AA31" s="37"/>
-    </row>
-    <row r="32" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="62"/>
-      <c r="C32" s="63"/>
-      <c r="D32" s="64"/>
-      <c r="E32" s="65"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="66"/>
-      <c r="H32" s="66"/>
-      <c r="I32" s="67"/>
-      <c r="J32" s="68"/>
-      <c r="K32" s="68"/>
-      <c r="L32" s="68"/>
-      <c r="M32" s="68"/>
-      <c r="N32" s="68"/>
-      <c r="O32" s="68"/>
-      <c r="P32" s="68"/>
-      <c r="Q32" s="68"/>
-      <c r="R32" s="68"/>
-      <c r="S32" s="61"/>
-      <c r="T32" s="69"/>
-      <c r="U32" s="69"/>
-      <c r="V32" s="69"/>
-      <c r="W32" s="53"/>
-      <c r="Y32" s="36"/>
-      <c r="Z32" s="37"/>
-      <c r="AA32" s="37"/>
-    </row>
-    <row r="33" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="70"/>
-      <c r="C33" s="71"/>
-      <c r="D33" s="72"/>
-      <c r="E33" s="73"/>
-      <c r="F33" s="74" t="s">
-        <v>4</v>
-      </c>
-      <c r="G33" s="75"/>
-      <c r="H33" s="75"/>
-      <c r="I33" s="76"/>
-      <c r="J33" s="77"/>
-      <c r="K33" s="77"/>
-      <c r="L33" s="77"/>
-      <c r="M33" s="78" t="s">
-        <v>35</v>
-      </c>
-      <c r="N33" s="77"/>
-      <c r="O33" s="78"/>
-      <c r="P33" s="77"/>
-      <c r="Q33" s="77"/>
-      <c r="R33" s="77"/>
-      <c r="S33" s="79"/>
-      <c r="T33" s="78"/>
-      <c r="U33" s="78"/>
-      <c r="V33" s="80"/>
-      <c r="W33" s="81"/>
-      <c r="Y33" s="36"/>
-      <c r="Z33" s="37"/>
-      <c r="AA33" s="37"/>
-    </row>
-    <row r="34" spans="2:27" s="35" customFormat="1" ht="22.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="82"/>
-      <c r="C34" s="38"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="40">
-        <v>1</v>
-      </c>
-      <c r="F34" s="156" t="s">
-        <v>64</v>
-      </c>
-      <c r="G34" s="157"/>
-      <c r="H34" s="157"/>
-      <c r="I34" s="41"/>
-      <c r="J34" s="148"/>
-      <c r="K34" s="42"/>
-      <c r="L34" s="42"/>
-      <c r="M34" s="42"/>
-      <c r="N34" s="42"/>
-      <c r="O34" s="42"/>
-      <c r="P34" s="42"/>
-      <c r="Q34" s="42"/>
-      <c r="R34" s="42"/>
-      <c r="S34" s="83"/>
-      <c r="T34" s="44"/>
-      <c r="U34" s="56"/>
-      <c r="V34" s="44"/>
-      <c r="W34" s="84"/>
-      <c r="Y34" s="36"/>
-      <c r="Z34" s="37"/>
-      <c r="AA34" s="37"/>
-    </row>
-    <row r="35" spans="2:27" s="35" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="82"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="40">
-        <v>2</v>
-      </c>
-      <c r="F35" s="158" t="s">
-        <v>65</v>
-      </c>
-      <c r="G35" s="159"/>
-      <c r="H35" s="159"/>
-      <c r="I35" s="41"/>
-      <c r="J35" s="147"/>
-      <c r="K35" s="42"/>
-      <c r="L35" s="42"/>
-      <c r="M35" s="42"/>
-      <c r="N35" s="42"/>
-      <c r="O35" s="42"/>
-      <c r="P35" s="42"/>
-      <c r="Q35" s="42"/>
-      <c r="R35" s="85"/>
-      <c r="S35" s="86"/>
-      <c r="T35" s="44"/>
-      <c r="U35" s="56"/>
-      <c r="V35" s="87"/>
-      <c r="W35" s="84"/>
-      <c r="Y35" s="36"/>
-      <c r="Z35" s="37"/>
-      <c r="AA35" s="37"/>
-    </row>
-    <row r="36" spans="2:27" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="B36" s="27"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="48">
-        <v>3</v>
-      </c>
-      <c r="F36" s="158"/>
-      <c r="G36" s="159"/>
-      <c r="H36" s="159"/>
-      <c r="I36" s="50"/>
-      <c r="J36" s="51"/>
-      <c r="K36" s="51"/>
-      <c r="L36" s="51"/>
-      <c r="M36" s="51"/>
-      <c r="N36" s="51"/>
-      <c r="O36" s="51"/>
-      <c r="P36" s="51"/>
-      <c r="Q36" s="51"/>
-      <c r="R36" s="51"/>
-      <c r="S36" s="43"/>
-      <c r="T36" s="88"/>
-      <c r="U36" s="44"/>
-      <c r="V36" s="56"/>
-      <c r="W36" s="89"/>
-      <c r="Y36" s="36"/>
-      <c r="Z36" s="37"/>
-      <c r="AA36" s="37"/>
-    </row>
-    <row r="37" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="27"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="47"/>
-      <c r="E37" s="48">
-        <v>4</v>
-      </c>
-      <c r="I37" s="50"/>
-      <c r="J37" s="51"/>
-      <c r="K37" s="51"/>
-      <c r="L37" s="51"/>
-      <c r="M37" s="51"/>
-      <c r="N37" s="51"/>
-      <c r="O37" s="51"/>
-      <c r="P37" s="51"/>
-      <c r="Q37" s="51"/>
-      <c r="R37" s="54"/>
-      <c r="S37" s="43"/>
-      <c r="T37" s="56"/>
-      <c r="U37" s="44"/>
-      <c r="V37" s="90"/>
-      <c r="W37" s="45"/>
-      <c r="Y37" s="36"/>
-      <c r="Z37" s="37"/>
-      <c r="AA37" s="37"/>
-    </row>
-    <row r="38" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="27"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="48">
-        <v>5</v>
-      </c>
-      <c r="I38" s="50"/>
-      <c r="J38" s="51"/>
-      <c r="K38" s="51"/>
-      <c r="L38" s="51"/>
-      <c r="M38" s="51"/>
-      <c r="N38" s="51"/>
-      <c r="O38" s="51"/>
-      <c r="P38" s="51"/>
-      <c r="Q38" s="51"/>
-      <c r="R38" s="51"/>
-      <c r="S38" s="52"/>
-      <c r="T38" s="44"/>
-      <c r="U38" s="44"/>
-      <c r="V38" s="44"/>
-      <c r="W38" s="53"/>
-      <c r="Y38" s="36"/>
-      <c r="Z38" s="37"/>
-      <c r="AA38" s="37"/>
-    </row>
-    <row r="39" spans="2:27" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="91"/>
-      <c r="C39" s="92"/>
-      <c r="D39" s="93"/>
-      <c r="E39" s="94"/>
-      <c r="F39" s="95"/>
-      <c r="G39" s="96"/>
-      <c r="H39" s="96"/>
-      <c r="I39" s="97"/>
-      <c r="J39" s="98"/>
-      <c r="K39" s="98"/>
-      <c r="L39" s="98"/>
-      <c r="M39" s="98"/>
-      <c r="N39" s="98"/>
-      <c r="O39" s="98"/>
-      <c r="P39" s="98"/>
-      <c r="Q39" s="98"/>
-      <c r="R39" s="98"/>
-      <c r="S39" s="97"/>
-      <c r="T39" s="98"/>
-      <c r="U39" s="98"/>
-      <c r="V39" s="99"/>
-      <c r="W39" s="100"/>
-      <c r="Y39" s="36"/>
-      <c r="Z39" s="37"/>
-      <c r="AA39" s="37"/>
-    </row>
-    <row r="40" spans="2:27" s="35" customFormat="1" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="101"/>
-      <c r="C40" s="102"/>
-      <c r="D40" s="103"/>
-      <c r="E40" s="104"/>
-      <c r="F40" s="105"/>
-      <c r="G40" s="106"/>
-      <c r="H40" s="107" t="s">
-        <v>5</v>
-      </c>
-      <c r="I40" s="108"/>
-      <c r="J40" s="109"/>
-      <c r="K40" s="109"/>
-      <c r="L40" s="109"/>
-      <c r="M40" s="109"/>
-      <c r="N40" s="109"/>
-      <c r="O40" s="109"/>
-      <c r="P40" s="109"/>
-      <c r="Q40" s="109"/>
-      <c r="R40" s="109"/>
-      <c r="S40" s="108"/>
-      <c r="T40" s="109"/>
-      <c r="U40" s="109"/>
-      <c r="V40" s="110"/>
-      <c r="W40" s="111"/>
-      <c r="Y40" s="36"/>
-      <c r="Z40" s="37"/>
-      <c r="AA40" s="37"/>
-    </row>
-    <row r="41" spans="2:27" s="35" customFormat="1" ht="4.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="112"/>
-      <c r="C41" s="113"/>
-      <c r="D41" s="114"/>
-      <c r="E41" s="115"/>
-      <c r="F41" s="116"/>
-      <c r="G41" s="116"/>
-      <c r="H41" s="116"/>
-      <c r="I41" s="117"/>
-      <c r="J41" s="118"/>
-      <c r="K41" s="118"/>
-      <c r="L41" s="118"/>
-      <c r="M41" s="118"/>
-      <c r="N41" s="118"/>
-      <c r="O41" s="118"/>
-      <c r="P41" s="118"/>
-      <c r="Q41" s="118"/>
-      <c r="R41" s="118"/>
-      <c r="S41" s="117"/>
-      <c r="T41" s="118"/>
-      <c r="U41" s="118"/>
-      <c r="V41" s="119"/>
-      <c r="W41" s="120"/>
-      <c r="X41" s="1"/>
-      <c r="Y41" s="36"/>
-      <c r="Z41" s="37"/>
-      <c r="AA41" s="37"/>
-    </row>
-    <row r="42" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="191"/>
-      <c r="C42" s="191"/>
-      <c r="D42" s="194"/>
-      <c r="F42" s="121"/>
-      <c r="G42" s="122"/>
-      <c r="H42" s="122"/>
-      <c r="I42" s="196" t="s">
-        <v>19</v>
-      </c>
-      <c r="J42" s="196" t="s">
-        <v>20</v>
-      </c>
-      <c r="K42" s="196" t="s">
-        <v>21</v>
-      </c>
-      <c r="L42" s="196" t="s">
-        <v>22</v>
-      </c>
-      <c r="M42" s="196" t="s">
-        <v>23</v>
-      </c>
-      <c r="N42" s="196" t="s">
-        <v>24</v>
-      </c>
-      <c r="O42" s="196" t="s">
-        <v>25</v>
-      </c>
-      <c r="P42" s="196" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q42" s="196" t="s">
-        <v>27</v>
-      </c>
-      <c r="R42" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="S42" s="200" t="s">
-        <v>14</v>
-      </c>
-      <c r="T42" s="203" t="s">
-        <v>15</v>
-      </c>
-      <c r="U42" s="203" t="s">
-        <v>16</v>
-      </c>
-      <c r="V42" s="203" t="s">
-        <v>18</v>
-      </c>
-      <c r="W42" s="213" t="s">
-        <v>17</v>
-      </c>
-      <c r="Y42" s="36"/>
-      <c r="Z42" s="37"/>
-      <c r="AA42" s="37"/>
-    </row>
-    <row r="43" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="192"/>
-      <c r="C43" s="192"/>
-      <c r="D43" s="194"/>
-      <c r="F43" s="123"/>
-      <c r="G43" s="122"/>
-      <c r="H43" s="122"/>
-      <c r="I43" s="196"/>
-      <c r="J43" s="196"/>
-      <c r="K43" s="196"/>
-      <c r="L43" s="196"/>
-      <c r="M43" s="196"/>
-      <c r="N43" s="196"/>
-      <c r="O43" s="196"/>
-      <c r="P43" s="196"/>
-      <c r="Q43" s="196"/>
-      <c r="R43" s="196"/>
-      <c r="S43" s="201"/>
-      <c r="T43" s="204"/>
-      <c r="U43" s="204"/>
-      <c r="V43" s="203"/>
-      <c r="W43" s="214"/>
-      <c r="Y43" s="36"/>
-      <c r="Z43" s="37"/>
-      <c r="AA43" s="37"/>
-    </row>
-    <row r="44" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="192"/>
-      <c r="C44" s="192"/>
-      <c r="D44" s="194"/>
-      <c r="F44" s="121"/>
-      <c r="G44" s="122"/>
-      <c r="H44" s="122"/>
-      <c r="I44" s="196"/>
-      <c r="J44" s="196"/>
-      <c r="K44" s="196"/>
-      <c r="L44" s="196"/>
-      <c r="M44" s="196"/>
-      <c r="N44" s="196"/>
-      <c r="O44" s="196"/>
-      <c r="P44" s="196"/>
-      <c r="Q44" s="196"/>
-      <c r="R44" s="196"/>
-      <c r="S44" s="201"/>
-      <c r="T44" s="204"/>
-      <c r="U44" s="204"/>
-      <c r="V44" s="203"/>
-      <c r="W44" s="214"/>
-      <c r="Z44" s="37"/>
-      <c r="AA44" s="37"/>
-    </row>
-    <row r="45" spans="2:27" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="192"/>
-      <c r="C45" s="192"/>
-      <c r="D45" s="194"/>
-      <c r="F45" s="124"/>
-      <c r="G45" s="122"/>
-      <c r="H45" s="122"/>
-      <c r="I45" s="197"/>
-      <c r="J45" s="197"/>
-      <c r="K45" s="197"/>
-      <c r="L45" s="197"/>
-      <c r="M45" s="197"/>
-      <c r="N45" s="197"/>
-      <c r="O45" s="197"/>
-      <c r="P45" s="197"/>
-      <c r="Q45" s="197"/>
-      <c r="R45" s="197"/>
-      <c r="S45" s="202"/>
-      <c r="T45" s="205"/>
-      <c r="U45" s="205"/>
-      <c r="V45" s="212"/>
-      <c r="W45" s="215"/>
-      <c r="Z45" s="2"/>
-      <c r="AA45" s="2"/>
-    </row>
-    <row r="46" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="192"/>
-      <c r="C46" s="192"/>
-      <c r="D46" s="194"/>
-      <c r="F46" s="124"/>
-      <c r="G46" s="124"/>
-      <c r="H46" s="124"/>
-      <c r="I46" s="125"/>
-      <c r="J46" s="126"/>
-      <c r="K46" s="126"/>
-      <c r="L46" s="126"/>
-      <c r="M46" s="126"/>
-      <c r="N46" s="126"/>
-      <c r="O46" s="126"/>
-      <c r="P46" s="126"/>
-      <c r="Q46" s="126"/>
-      <c r="R46" s="126"/>
-      <c r="S46" s="126"/>
-      <c r="T46" s="126"/>
-      <c r="U46" s="126"/>
-      <c r="V46" s="126"/>
-      <c r="W46" s="127"/>
-      <c r="Z46" s="37"/>
-      <c r="AA46" s="37"/>
-    </row>
-    <row r="47" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="192"/>
-      <c r="C47" s="192"/>
-      <c r="D47" s="194"/>
-      <c r="E47" s="128"/>
-      <c r="F47" s="124"/>
-      <c r="G47" s="123"/>
-      <c r="H47" s="123"/>
-      <c r="I47" s="129"/>
-      <c r="J47" s="130"/>
-      <c r="K47" s="130"/>
-      <c r="L47" s="130"/>
-      <c r="M47" s="130"/>
-      <c r="N47" s="130"/>
-      <c r="O47" s="130"/>
-      <c r="P47" s="130"/>
-      <c r="Q47" s="130"/>
-      <c r="R47" s="130"/>
-      <c r="S47" s="130"/>
-      <c r="T47" s="130"/>
-      <c r="U47" s="130"/>
-      <c r="V47" s="130"/>
-      <c r="W47" s="131"/>
-      <c r="Z47" s="2"/>
-      <c r="AA47" s="2"/>
-    </row>
-    <row r="48" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="192"/>
-      <c r="C48" s="192"/>
-      <c r="D48" s="194"/>
-      <c r="F48" s="121"/>
-      <c r="G48" s="123"/>
-      <c r="H48" s="123"/>
-      <c r="I48" s="129"/>
-      <c r="J48" s="130"/>
-      <c r="K48" s="130"/>
-      <c r="L48" s="130"/>
-      <c r="M48" s="130"/>
-      <c r="N48" s="130"/>
-      <c r="O48" s="130"/>
-      <c r="P48" s="130"/>
-      <c r="Q48" s="130"/>
-      <c r="R48" s="130"/>
-      <c r="S48" s="130"/>
-      <c r="T48" s="130"/>
-      <c r="U48" s="130"/>
-      <c r="V48" s="130"/>
-      <c r="W48" s="131"/>
-      <c r="Z48" s="37"/>
-      <c r="AA48" s="37"/>
-    </row>
-    <row r="49" spans="2:27" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B49" s="192"/>
-      <c r="C49" s="192"/>
-      <c r="D49" s="194"/>
-      <c r="F49" s="121"/>
-      <c r="G49" s="123"/>
-      <c r="H49" s="132"/>
-      <c r="I49" s="129"/>
-      <c r="J49" s="130"/>
-      <c r="K49" s="130"/>
-      <c r="L49" s="130"/>
-      <c r="M49" s="130"/>
-      <c r="N49" s="130"/>
-      <c r="O49" s="130"/>
-      <c r="P49" s="130"/>
-      <c r="Q49" s="130"/>
-      <c r="R49" s="130"/>
-      <c r="S49" s="130"/>
-      <c r="T49" s="130"/>
-      <c r="U49" s="130"/>
-      <c r="V49" s="130"/>
-      <c r="W49" s="131"/>
-      <c r="Z49" s="2"/>
-      <c r="AA49" s="2"/>
-    </row>
-    <row r="50" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="192"/>
-      <c r="C50" s="192"/>
-      <c r="D50" s="194"/>
-      <c r="F50" s="121"/>
-      <c r="G50" s="121"/>
-      <c r="H50" s="121"/>
-      <c r="I50" s="129"/>
-      <c r="J50" s="130"/>
-      <c r="K50" s="130"/>
-      <c r="L50" s="130"/>
-      <c r="M50" s="130"/>
-      <c r="N50" s="130"/>
-      <c r="O50" s="130"/>
-      <c r="P50" s="130"/>
-      <c r="Q50" s="130"/>
-      <c r="R50" s="130"/>
-      <c r="S50" s="130"/>
-      <c r="T50" s="130"/>
-      <c r="U50" s="130"/>
-      <c r="V50" s="130"/>
-      <c r="W50" s="131"/>
-      <c r="Z50" s="37"/>
-      <c r="AA50" s="37"/>
-    </row>
-    <row r="51" spans="2:27" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="192"/>
-      <c r="C51" s="192"/>
-      <c r="D51" s="194"/>
-      <c r="F51" s="133"/>
-      <c r="I51" s="129"/>
-      <c r="J51" s="130"/>
-      <c r="K51" s="130"/>
-      <c r="L51" s="130"/>
-      <c r="M51" s="130"/>
-      <c r="N51" s="130"/>
-      <c r="O51" s="130"/>
-      <c r="P51" s="130"/>
-      <c r="Q51" s="130"/>
-      <c r="R51" s="130"/>
-      <c r="S51" s="130"/>
-      <c r="T51" s="130"/>
-      <c r="U51" s="130"/>
-      <c r="V51" s="130"/>
-      <c r="W51" s="131"/>
-      <c r="Z51" s="2"/>
-      <c r="AA51" s="2"/>
-    </row>
-    <row r="52" spans="2:27" ht="50.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="192"/>
-      <c r="C52" s="192"/>
-      <c r="D52" s="194"/>
-      <c r="E52" s="135"/>
-      <c r="F52" s="135"/>
-      <c r="G52" s="135"/>
-      <c r="H52" s="135"/>
-      <c r="I52" s="136"/>
-      <c r="J52" s="137"/>
-      <c r="K52" s="137"/>
-      <c r="L52" s="137"/>
-      <c r="M52" s="137"/>
-      <c r="N52" s="137"/>
-      <c r="O52" s="137"/>
-      <c r="P52" s="137"/>
-      <c r="Q52" s="137"/>
-      <c r="R52" s="137"/>
-      <c r="S52" s="137"/>
-      <c r="T52" s="137"/>
-      <c r="U52" s="137"/>
-      <c r="V52" s="137"/>
-      <c r="W52" s="138"/>
-      <c r="Z52" s="134"/>
-      <c r="AA52" s="134"/>
-    </row>
-    <row r="53" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="192"/>
-      <c r="C53" s="192"/>
-      <c r="D53" s="194"/>
-      <c r="E53" s="206"/>
-      <c r="F53" s="206"/>
-      <c r="G53" s="206"/>
-      <c r="H53" s="206"/>
-      <c r="I53" s="206"/>
-      <c r="J53" s="206"/>
-      <c r="K53" s="206"/>
-      <c r="L53" s="206"/>
-      <c r="M53" s="206"/>
-      <c r="N53" s="206"/>
-      <c r="O53" s="206"/>
-      <c r="P53" s="206"/>
-      <c r="Q53" s="206"/>
-      <c r="R53" s="206"/>
-      <c r="S53" s="206"/>
-      <c r="T53" s="206"/>
-      <c r="U53" s="206"/>
-      <c r="V53" s="206"/>
-      <c r="W53" s="207"/>
-    </row>
-    <row r="54" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="192"/>
-      <c r="C54" s="192"/>
-      <c r="D54" s="194"/>
-      <c r="E54" s="208"/>
-      <c r="F54" s="208"/>
-      <c r="G54" s="208"/>
-      <c r="H54" s="208"/>
-      <c r="I54" s="208"/>
-      <c r="J54" s="208"/>
-      <c r="K54" s="208"/>
-      <c r="L54" s="208"/>
-      <c r="M54" s="208"/>
-      <c r="N54" s="208"/>
-      <c r="O54" s="208"/>
-      <c r="P54" s="208"/>
-      <c r="Q54" s="208"/>
-      <c r="R54" s="208"/>
-      <c r="S54" s="208"/>
-      <c r="T54" s="208"/>
-      <c r="U54" s="208"/>
-      <c r="V54" s="208"/>
-      <c r="W54" s="209"/>
-    </row>
-    <row r="55" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="192"/>
-      <c r="C55" s="192"/>
-      <c r="D55" s="194"/>
-      <c r="E55" s="208"/>
-      <c r="F55" s="208"/>
-      <c r="G55" s="208"/>
-      <c r="H55" s="208"/>
-      <c r="I55" s="208"/>
-      <c r="J55" s="208"/>
-      <c r="K55" s="208"/>
-      <c r="L55" s="208"/>
-      <c r="M55" s="208"/>
-      <c r="N55" s="208"/>
-      <c r="O55" s="208"/>
-      <c r="P55" s="208"/>
-      <c r="Q55" s="208"/>
-      <c r="R55" s="208"/>
-      <c r="S55" s="208"/>
-      <c r="T55" s="208"/>
-      <c r="U55" s="208"/>
-      <c r="V55" s="208"/>
-      <c r="W55" s="209"/>
-    </row>
-    <row r="56" spans="2:27" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="193"/>
-      <c r="C56" s="193"/>
-      <c r="D56" s="195"/>
-      <c r="E56" s="198"/>
-      <c r="F56" s="198"/>
-      <c r="G56" s="198"/>
-      <c r="H56" s="198"/>
-      <c r="I56" s="198"/>
-      <c r="J56" s="198"/>
-      <c r="K56" s="198"/>
-      <c r="L56" s="198"/>
-      <c r="M56" s="198"/>
-      <c r="N56" s="198"/>
-      <c r="O56" s="198"/>
-      <c r="P56" s="198"/>
-      <c r="Q56" s="198"/>
-      <c r="R56" s="198"/>
-      <c r="S56" s="198"/>
-      <c r="T56" s="198"/>
-      <c r="U56" s="198"/>
-      <c r="V56" s="198"/>
-      <c r="W56" s="199"/>
-    </row>
-    <row r="58" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="K58" s="139" t="s">
-        <v>7</v>
-      </c>
-      <c r="L58" s="139" t="s">
-        <v>6</v>
-      </c>
-      <c r="M58" s="139" t="s">
-        <v>9</v>
-      </c>
-      <c r="N58" s="139" t="s">
-        <v>8</v>
-      </c>
-      <c r="O58" s="140"/>
-      <c r="P58" s="140"/>
-      <c r="Q58" s="140"/>
-      <c r="R58" s="140"/>
-      <c r="S58" s="141" t="s">
-        <v>11</v>
-      </c>
-      <c r="T58" s="210" t="s">
-        <v>29</v>
-      </c>
-      <c r="U58" s="211"/>
-      <c r="V58" s="140"/>
-      <c r="W58" s="140"/>
-      <c r="X58" s="140"/>
-      <c r="Y58" s="140"/>
-      <c r="Z58" s="140"/>
-      <c r="AA58" s="140"/>
-    </row>
-    <row r="59" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="J59" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K59" s="142" t="s">
-        <v>7</v>
-      </c>
-      <c r="L59" s="142" t="s">
-        <v>6</v>
-      </c>
-      <c r="M59" s="142" t="s">
-        <v>9</v>
-      </c>
-      <c r="N59" s="142" t="s">
-        <v>8</v>
-      </c>
-      <c r="O59" s="57"/>
-      <c r="P59" s="57"/>
-      <c r="Q59" s="57"/>
-      <c r="R59" s="57"/>
-      <c r="S59" s="143" t="s">
-        <v>12</v>
-      </c>
-      <c r="T59" s="210" t="s">
-        <v>30</v>
-      </c>
-      <c r="U59" s="211"/>
-      <c r="V59" s="57"/>
-      <c r="W59" s="57"/>
-      <c r="X59" s="57"/>
-      <c r="Y59" s="57"/>
-      <c r="Z59" s="57"/>
-      <c r="AA59" s="57"/>
-    </row>
-    <row r="60" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="S60" s="144" t="s">
-        <v>13</v>
-      </c>
-      <c r="T60" s="210" t="s">
-        <v>31</v>
-      </c>
-      <c r="U60" s="211"/>
-      <c r="Y60" s="1"/>
-      <c r="Z60" s="1"/>
-      <c r="AA60" s="1"/>
-    </row>
-    <row r="61" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="Y61" s="1"/>
-      <c r="Z61" s="1"/>
-      <c r="AA61" s="1"/>
-    </row>
-    <row r="62" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="K62" s="145"/>
-      <c r="L62" s="146" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="63" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="K63" s="147"/>
-      <c r="L63" s="146" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="64" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="K64" s="148"/>
-      <c r="L64" s="146" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="56">
-    <mergeCell ref="T60:U60"/>
-    <mergeCell ref="E55:W55"/>
-    <mergeCell ref="U42:U45"/>
-    <mergeCell ref="L42:L45"/>
-    <mergeCell ref="M42:M45"/>
-    <mergeCell ref="N42:N45"/>
-    <mergeCell ref="O42:O45"/>
-    <mergeCell ref="P42:P45"/>
-    <mergeCell ref="Q42:Q45"/>
-    <mergeCell ref="V42:V45"/>
-    <mergeCell ref="W42:W45"/>
-    <mergeCell ref="E53:W53"/>
-    <mergeCell ref="E54:W54"/>
-    <mergeCell ref="T58:U58"/>
-    <mergeCell ref="T59:U59"/>
+  <mergeCells count="52">
+    <mergeCell ref="R55:S55"/>
+    <mergeCell ref="E50:U50"/>
+    <mergeCell ref="S37:S40"/>
+    <mergeCell ref="L37:L40"/>
+    <mergeCell ref="M37:M40"/>
+    <mergeCell ref="N37:N40"/>
+    <mergeCell ref="O37:O40"/>
+    <mergeCell ref="P37:P40"/>
+    <mergeCell ref="T37:T40"/>
+    <mergeCell ref="U37:U40"/>
+    <mergeCell ref="E48:U48"/>
+    <mergeCell ref="E49:U49"/>
+    <mergeCell ref="R53:S53"/>
+    <mergeCell ref="R54:S54"/>
+    <mergeCell ref="K37:K40"/>
+    <mergeCell ref="E51:U51"/>
+    <mergeCell ref="Q37:Q40"/>
+    <mergeCell ref="R37:R40"/>
+    <mergeCell ref="B37:B51"/>
+    <mergeCell ref="C37:C51"/>
+    <mergeCell ref="D37:D51"/>
+    <mergeCell ref="I37:I40"/>
+    <mergeCell ref="J37:J40"/>
+    <mergeCell ref="E3:U4"/>
+    <mergeCell ref="F12:H12"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="I5:R5"/>
-    <mergeCell ref="S5:W5"/>
-    <mergeCell ref="B42:B56"/>
-    <mergeCell ref="C42:C56"/>
-    <mergeCell ref="D42:D56"/>
-    <mergeCell ref="I42:I45"/>
-    <mergeCell ref="J42:J45"/>
-    <mergeCell ref="K42:K45"/>
-    <mergeCell ref="E56:W56"/>
-    <mergeCell ref="R42:R45"/>
-    <mergeCell ref="S42:S45"/>
-    <mergeCell ref="T42:T45"/>
+    <mergeCell ref="I5:P5"/>
+    <mergeCell ref="Q5:U5"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="F9:H9"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="F8:H8"/>
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="F11:H11"/>
     <mergeCell ref="F13:H13"/>
-    <mergeCell ref="E3:W4"/>
-    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="F25:H25"/>
     <mergeCell ref="B6:D9"/>
     <mergeCell ref="B10:D13"/>
     <mergeCell ref="B14:D23"/>
@@ -5792,20 +5693,14 @@
     <mergeCell ref="F15:H15"/>
     <mergeCell ref="F16:H16"/>
     <mergeCell ref="F17:H17"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="F25:H25"/>
   </mergeCells>
-  <conditionalFormatting sqref="B41:D41">
+  <phoneticPr fontId="18" type="noConversion"/>
+  <conditionalFormatting sqref="B36:D36">
     <cfRule type="cellIs" dxfId="28" priority="79" stopIfTrue="1" operator="notEqual">
       <formula>""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H59:I59 V59:AA59">
+  <conditionalFormatting sqref="H54:I54 T54:Y54">
     <cfRule type="cellIs" dxfId="27" priority="83" stopIfTrue="1" operator="equal">
       <formula>"G"</formula>
     </cfRule>
@@ -5816,7 +5711,7 @@
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:R16 I17:K17 M17:R17 I18:R19 I20:M20 O20:R20 N20:N21 I21:L28">
+  <conditionalFormatting sqref="I17:K17 M17:P17 I18:P19 I20:M20 O20:P20 N20:N21 I21:L26 I6:P16">
     <cfRule type="cellIs" dxfId="24" priority="70" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
@@ -5827,12 +5722,12 @@
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I31:R33 I34:I35 K34:R35 I36:R40">
+  <conditionalFormatting sqref="I27:P28 I29:I31 K29:P31 I32:P35">
     <cfRule type="cellIs" dxfId="21" priority="33" stopIfTrue="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I31:R33 I34:I35 K34:R35 I36:R41">
+  <conditionalFormatting sqref="I27:P28 I29:I31 K29:P31 I32:P36">
     <cfRule type="cellIs" dxfId="20" priority="31" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
@@ -5840,12 +5735,12 @@
       <formula>"C"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I41:R41">
+  <conditionalFormatting sqref="I36:P36">
     <cfRule type="cellIs" dxfId="18" priority="82" stopIfTrue="1" operator="equal">
       <formula>"L"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M21 R21:R30 M22:N23 N27:P28 I29:P29 I30:O30 Q30">
+  <conditionalFormatting sqref="M21 M22:N23">
     <cfRule type="cellIs" dxfId="17" priority="73" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
@@ -5867,7 +5762,7 @@
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M59:R59">
+  <conditionalFormatting sqref="M54:P54">
     <cfRule type="cellIs" dxfId="11" priority="46" stopIfTrue="1" operator="equal">
       <formula>"G"</formula>
     </cfRule>
@@ -5889,18 +5784,7 @@
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q21:Q28">
-    <cfRule type="cellIs" dxfId="5" priority="22" stopIfTrue="1" operator="equal">
-      <formula>"S"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="23" stopIfTrue="1" operator="equal">
-      <formula>"C"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="24" stopIfTrue="1" operator="equal">
-      <formula>"D"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S41:W41">
+  <conditionalFormatting sqref="Q36:U36">
     <cfRule type="cellIs" dxfId="2" priority="76" stopIfTrue="1" operator="equal">
       <formula>"A"</formula>
     </cfRule>

</xml_diff>